<commit_message>
Able to connect playwright and selenium on same chrome profile, now able to use simplify
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF21"/>
+  <dimension ref="A1:AF31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2263,7 +2263,7 @@
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr">
@@ -2604,7 +2604,7 @@
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr">
@@ -4131,6 +4131,1766 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>4454012661</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>dII1y5WGyKGOqqap+dwppA==</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Hqan1SC6SBVwlDMjIWeHxQ==</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/ai-product-engineer-at-alexander-chapman-4454012661?position=7&amp;pageNum=0&amp;refId=Hqan1SC6SBVwlDMjIWeHxQ%3D%3D&amp;trackingId=dII1y5WGyKGOqqap%2BdwppA%3D%3D</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>AI Product Engineer</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Alexander Chapman</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://uk.linkedin.com/company/alexander-chapman?trk=public_jobs_jserp-result_job-search-card-subtitle</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>https://media.licdn.com/dms/image/v2/C4E0BAQHetz_sr_qHBQ/company-logo_100_100/company-logo_100_100/0/1647822869660/alexander_chapman_logo?e=2147483647&amp;v=beta&amp;t=fXf23KD1xm92km0--__xsbUDUOxFVSIlMPe2k053cE0</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>California, United States</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Connect for more:&lt;/strong&gt; https://www.linkedin.com/in/arianit-krasniqi-b6ba66388/&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;I'm working with a fast-growing startup building an &lt;strong&gt;AI platform that runs business operations autonomously&lt;/strong&gt; through &lt;strong&gt;multi-agent systems&lt;/strong&gt;. They are seeking a &lt;strong&gt;Product Engineer&lt;/strong&gt; to own and ship &lt;strong&gt;LLM-powered features end-to-end&lt;/strong&gt;, directly impacting how enterprises operate.&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;This is a highly &lt;strong&gt;builder-first role&lt;/strong&gt;, where engineers take full ownership from &lt;strong&gt;customer problem → design → production → iteration&lt;/strong&gt;, working closely with users and shipping continuously. The focus is on building &lt;strong&gt;agent systems&lt;/strong&gt; that execute workflows like &lt;strong&gt;OKRs, reporting cadences, and operational playbooks&lt;/strong&gt;, while ensuring &lt;strong&gt;enterprise-grade reliability&lt;/strong&gt;.&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;Engineers will design and implement &lt;strong&gt;multi-agent architectures&lt;/strong&gt;, make decisions around &lt;strong&gt;model selection, orchestration, and evaluation&lt;/strong&gt;, and build &lt;strong&gt;chat-native product experiences&lt;/strong&gt; used daily by customers. The role combines &lt;strong&gt;systems thinking with product intuition&lt;/strong&gt;, requiring strong judgment on tradeoffs between capability, reliability, and user impact.&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;Ideal candidates have &lt;strong&gt;2–5 years of experience&lt;/strong&gt;, strong skills in &lt;strong&gt;Python&lt;/strong&gt; and familiarity with &lt;strong&gt;React/Next.js&lt;/strong&gt;, and hands-on experience shipping &lt;strong&gt;LLM or agent-based systems in production&lt;/strong&gt;. They are fast-moving, customer-focused builders who use &lt;strong&gt;AI tools daily&lt;/strong&gt;, iterate quickly in production, and thrive in &lt;strong&gt;high-ownership, early-stage environments&lt;/strong&gt;.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Connect for more: https://www.linkedin.com/in/arianit-krasniqi-b6ba66388/
+I'm working with a fast-growing startup building an AI platform that runs business operations autonomously through multi-agent systems. They are seeking a Product Engineer to own and ship LLM-powered features end-to-end, directly impacting how enterprises operate.
+This is a highly builder-first role, where engineers take full ownership from customer problem → design → production → iteration, working closely with users and shipping continuously. The focus is on building agent systems that execute workflows like OKRs, reporting cadences, and operational playbooks, while ensuring enterprise-grade reliability.
+Engineers will design and implement multi-agent architectures, make decisions around model selection, orchestration, and evaluation, and build chat-native product experiences used daily by customers. The role combines systems thinking with product intuition, requiring strong judgment on tradeoffs between capability, reliability, and user impact.
+Ideal candidates have 2–5 years of experience, strong skills in Python and familiarity with React/Next.js, and hands-on experience shipping LLM or agent-based systems in production. They are fast-moving, customer-focused builders who use AI tools daily, iterate quickly in production, and thrive in high-ownership, early-stage environments.</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Associate</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Software Development</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?position=1&amp;pageNum=0&amp;keywords=AI+Engineer&amp;location=United+States&amp;distance=0&amp;f_TPR=r86400</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>{'type': 'PostalAddress', 'addressLocality': 'London', 'addressCountry': 'gb'}</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>http://www.alexanderchapmanltd.com</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Matching excellence. </t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alexander Chapman is a leading global search firm specializing in comprehensive staffing and talent management solutions tailored to the unique needs of local, regional, national, and international businesses. With a dedicated focus on niche recruiting expertise and expert project management, Alexander Chapman excels in providing innovative solutions within the Finance sectors.
+</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>2026-08-14 05:10:51</t>
+        </is>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>Arianit Krasniqi</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr"/>
+      <c r="AE22" t="inlineStr">
+        <is>
+          <t>https://static.licdn.com/aero-v1/sc/h/9c8pery4andzj6ohjkjp54ma2</t>
+        </is>
+      </c>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/arianit-krasniqi-b6ba66388</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>4439922787</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>sKIn5g4B7M3fkzMKgR8m5g==</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Hqan1SC6SBVwlDMjIWeHxQ==</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/artificial-intelligence-engineer-at-neubird-ai-4439922787?position=8&amp;pageNum=0&amp;refId=Hqan1SC6SBVwlDMjIWeHxQ%3D%3D&amp;trackingId=sKIn5g4B7M3fkzMKgR8m5g%3D%3D</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence Engineer</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>NeuBird AI</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/neubird-ai?trk=public_jobs_jserp-result_job-search-card-subtitle</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://media.licdn.com/dms/image/v2/D560BAQF6OENzsfBHaQ/company-logo_100_100/B56ZwGcOhMHcAQ-/0/1769634589064/neubird_ai_logo?e=2147483647&amp;v=beta&amp;t=0YlYZc_RW7iV6oiiAEdYX3Q-CTVcdsCFWaZGYXB5ETQ</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>California, United States</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Job Description:&lt;/strong&gt;&lt;/p&gt;&lt;p&gt;As an AI engineer, you will be involved in model training, deployment, and maintenance. You will work with RLHF and fine-tuning of LLMs. This role requires a blend of analytical skills, creativity, and strong AI domain knowledge. This role is critical in delivering an enterprise experience with LLMs.&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;&lt;strong&gt;&lt;br&gt;&lt;br&gt;Responsibilitie&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;s:Lead the development and customization of large-scale language models that drive the NeuBird AI platfor&lt;/li&gt;&lt;li&gt;m.Implement and experiment with RLHF to enhance model performance and decision-makin&lt;/li&gt;&lt;li&gt;g.Collaborate with cross-functional teams to integrate language models into various applications and platform&lt;/li&gt;&lt;li&gt;s.Work on model fine-tuning, performance optimization, and continuous improvemen&lt;/li&gt;&lt;li&gt;t.Stay up-to-date with the latest research and trends in language modeling and RLH&lt;/li&gt;&lt;li&gt;F.Contribute to research projects and technical publication&lt;/li&gt;&lt;li&gt;s.Participate in code reviews and mentorship of junior engineer&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;&lt;strong&gt;s.&lt;br&gt;&lt;br&gt;Qualificati&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;ons:Bachelor's or Master's degree in Computer Science, Machine Learning, or a related f&lt;/li&gt;&lt;li&gt;ieldExperience with model training, deploying, and maintena&lt;/li&gt;&lt;li&gt;nce.Strong knowledge of reinforced feedback techniques and reinforcement learn&lt;/li&gt;&lt;li&gt;ing.Proficiency in frameworks like PyTorch, TensorFlow, or simi&lt;/li&gt;&lt;li&gt;lar.Familiarity with NLP, text generation, and language understand&lt;/li&gt;&lt;li&gt;ing.Strong problem-solving skills and a passion for addressing complex AI challen&lt;/li&gt;&lt;li&gt;ges.Excellent communication and collaboration abilit&lt;/li&gt;&lt;li&gt;ies.Self-motivated and eager to stay at the forefront of AI advanceme&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;nts.</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Job Description:
+As an AI engineer, you will be involved in model training, deployment, and maintenance. You will work with RLHF and fine-tuning of LLMs. This role requires a blend of analytical skills, creativity, and strong AI domain knowledge. This role is critical in delivering an enterprise experience with LLMs.
+Responsibilitie
+- s:Lead the development and customization of large-scale language models that drive the NeuBird AI platfor
+- m.Implement and experiment with RLHF to enhance model performance and decision-makin
+- g.Collaborate with cross-functional teams to integrate language models into various applications and platform
+- s.Work on model fine-tuning, performance optimization, and continuous improvemen
+- t.Stay up-to-date with the latest research and trends in language modeling and RLH
+- F.Contribute to research projects and technical publication
+- s.Participate in code reviews and mentorship of junior engineer
+s.
+Qualificati
+- ons:Bachelor's or Master's degree in Computer Science, Machine Learning, or a related f
+- ieldExperience with model training, deploying, and maintena
+- nce.Strong knowledge of reinforced feedback techniques and reinforcement learn
+- ing.Proficiency in frameworks like PyTorch, TensorFlow, or simi
+- lar.Familiarity with NLP, text generation, and language understand
+- ing.Strong problem-solving skills and a passion for addressing complex AI challen
+- ges.Excellent communication and collaboration abilit
+- ies.Self-motivated and eager to stay at the forefront of AI advanceme
+nts.</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Entry level</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>IT System Custom Software Development</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?position=1&amp;pageNum=0&amp;keywords=AI+Engineer&amp;location=United+States&amp;distance=0&amp;f_TPR=r86400</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>{'type': 'PostalAddress', 'streetAddress': '2000 Broadway St', 'addressLocality': 'Redwood City', 'addressRegion': 'California', 'postalCode': '94063', 'addressCountry': 'US'}</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>https://neubird.ai</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>Autonomous production operations. 
+Prevent issues. Resolve in minutes. Operate autonomously.</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Production ops agent for modern engineering teams. Prevent issues before impact, resolve incidents in minutes, and operate production systems autonomously.
+Built for enterprise SRE, platform, DevOps, and on-call teams, NeuBird AI applies advanced context engineering and deep domain expertise to correlate telemetry, surface risks early, and automate root cause analysis securely across hybrid cloud environments.
+</t>
+        </is>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>2026-08-14 05:10:51</t>
+        </is>
+      </c>
+      <c r="AC23" t="inlineStr"/>
+      <c r="AD23" t="inlineStr"/>
+      <c r="AE23" t="inlineStr"/>
+      <c r="AF23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>4454304447</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>aH1wKYh1EjTn88dx66XmPQ==</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Hqan1SC6SBVwlDMjIWeHxQ==</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/ai-developer-at-booz-allen-hamilton-4454304447?position=9&amp;pageNum=0&amp;refId=Hqan1SC6SBVwlDMjIWeHxQ%3D%3D&amp;trackingId=aH1wKYh1EjTn88dx66XmPQ%3D%3D</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>AI Developer</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Booz Allen Hamilton</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/booz-allen-hamilton?trk=public_jobs_jserp-result_job-search-card-subtitle</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://media.licdn.com/dms/image/v2/D4E0BAQFXBzVcVDSTOQ/company-logo_100_100/company-logo_100_100/0/1737465459820/booz_allen_hamilton_logo?e=2147483647&amp;v=beta&amp;t=SswDqk5ZXqP0jtQgXL12ktHuwfRb0zf8se42kJe-lFM</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Arlington, VA</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>&lt;strong&gt;Job Number: R0246928&lt;br&gt;&lt;br&gt;&lt;/strong&gt;AI Developer&lt;br&gt;&lt;br&gt;&lt;strong&gt;The Opportunity: &lt;br&gt;&lt;br&gt;&lt;/strong&gt;As an experienced AI engineer, you know that AI systems are critical to understanding and processing massive datasets in an organization. Your ability to conduct statistical analyses on business processes using ML techniques makes you an integral part of delivering a customer-focused solution. We need your technical knowledge and desire to solve problems to support optimizing organizational efficiency. As an AI Developer on our Air Power team, you’ll train, test, deploy, and maintain models that learn from data.&lt;br&gt;&lt;br&gt;In this role, you’ll own and define the direction of mission-critical solutions by applying cutting-edge Agentic frameworks. You’ll be part of a large community of AI professionals across the company and collaborate with data engineers, data scientists, solutions architects, and product owners to deliver world-class solutions to transform how the Air Force manages its day-to-day business. Your skills and extensive technical expertise will guide clients as they navigate the landscape of Agentic Frameworks.&lt;br&gt;&lt;br&gt;Join us. The world can’t wait.&lt;br&gt;&lt;br&gt;&lt;strong&gt;You Have:&lt;br&gt;&lt;br&gt;&lt;/strong&gt;&lt;ul&gt;&lt;li&gt;2+ years of experience building production-grade software in Python, TypeScript, or Java with APIs and data services, including FastAPI, Flask, REST, GraphQL, or SQL&lt;/li&gt;&lt;li&gt;Experience developing and deploying AI-enabled applications such as LLMs, RAG, and agentic workflows to solve mission problems&lt;/li&gt;&lt;li&gt;Ability to design event-driven integrations and workflow automation such as asynchronous messaging or audit logging to move from insight to action&lt;/li&gt;&lt;li&gt;Ability to implement MLOps or DevSecOps practices such as CI/CD, containerization, automated testing, or model evaluation&lt;/li&gt;&lt;li&gt;Secret clearance&lt;/li&gt;&lt;li&gt;Bachelor’s degree in Mathematics, Computer Science, Software Engineering, or Data Science&lt;br&gt;&lt;br&gt;&lt;br&gt;&lt;/li&gt;&lt;/ul&gt;&lt;strong&gt;Nice If You Have:&lt;br&gt;&lt;br&gt;&lt;/strong&gt;&lt;ul&gt;&lt;li&gt;Experience working with geospatial or 3D data, including point clouds, LiDAR, or photogrammetry, or digital-twin or facility and asset data models&lt;/li&gt;&lt;li&gt;Experience integrating sensor streams or IoT telemetry and edge-to-cloud data flows such as Kafka, NATS, RabbitMQ, or equivalent for asset monitoring and situational awareness&lt;/li&gt;&lt;li&gt;Experience deploying software and data or ML pipelines in disconnected, air-gapped, or classified environments&lt;/li&gt;&lt;li&gt;Experience with cross-domain data handling constraints&lt;/li&gt;&lt;li&gt;Experience with RMF or STIG-aligned delivery&lt;/li&gt;&lt;li&gt;Experience with AI-assisted software development tools and practices such as code copilots, automated tests, or secure-by-design patterns to increase delivery velocity responsibly&lt;/li&gt;&lt;li&gt;TS/SCI clearance&lt;br&gt;&lt;br&gt;&lt;br&gt;&lt;/li&gt;&lt;/ul&gt;&lt;strong&gt;Clearance:&lt;/strong&gt; &lt;br&gt;&lt;br&gt;Applicants selected will be subject to a security investigation and may need to meet eligibility requirements for access to classified information; Secret clearance is required.&lt;br&gt;&lt;br&gt;&lt;strong&gt;Compensation&lt;br&gt;&lt;br&gt;&lt;/strong&gt;At Booz Allen, we celebrate your contributions, provide you with opportunities and choices, and support your total well-being. Our offerings include health, life, disability, financial, and retirement benefits, as well as paid leave, professional development, tuition assistance, work-life programs, and dependent care. Our recognition awards program acknowledges employees for exceptional performance and superior demonstration of our values. Full-time and part-time employees working at least 20 hours a week on a regular basis are eligible to participate in Booz Allen’s benefit programs. Individuals that do not meet the threshold are only eligible for select offerings, not inclusive of health benefits. We encourage you to learn more about our total benefits by visiting the Resource page on our Careers site and reviewing Our Employee Benefits page.&lt;br&gt;&lt;br&gt;Salary at Booz Allen is determined by various factors, including but not limited to location, the individual’s particular combination of education, knowledge, skills, competencies, and experience, as well as contract-specific affordability and organizational requirements. The projected compensation range for this position is $77,500.00 to $176,000.00 (annualized USD). The estimate displayed represents the typical salary range for this position and is just one component of Booz Allen’s total compensation package for employees. This posting will close within 90 days from the Posting Date.&lt;br&gt;&lt;br&gt;&lt;strong&gt;Identity Statement&lt;br&gt;&lt;br&gt;&lt;/strong&gt;As part of the hiring process, we will ask you to complete an identity verification process that leverages advanced biometrics and artificial intelligence to ensure authenticity and protect against identity fraud. You are expected to be on camera during interviews and assessments. We reserve the right to take your picture to verify your identity and prevent fraud.&lt;br&gt;&lt;br&gt;&lt;strong&gt;Candidate AI Usage Policy&lt;br&gt;&lt;br&gt;&lt;/strong&gt;AI is a part of our daily work at Booz Allen, and we are committed to the responsible and ethical use of AI tools. However, we want to ensure a fair candidate process based on &lt;strong&gt;your &lt;/strong&gt;own skills and knowledge. As part of this commitment, the use of artificial intelligence (AI) or other tools to assist with responses during interviews (whether in-person or virtual) is prohibited &lt;strong&gt;unless permission is explicitly provided&lt;/strong&gt;.&lt;br&gt;&lt;br&gt;&lt;strong&gt;Work Model&lt;br&gt;&lt;br&gt;&lt;/strong&gt;Our people-first culture prioritizes the benefits of collaboration, whether it occurs in person or virtually. To support engagement and effective communication, employees working virtually are generally expected to have their cameras on during meetings.&lt;br&gt;&lt;br&gt;&lt;ul&gt;&lt;li&gt;Remote: If this position is listed as remote, there may still be occasions when you are required to work in person at a Booz Allen or customer facility.&lt;/li&gt;&lt;li&gt;Hybrid: If this position is listed as hybrid, you will be expected to work from a Booz Allen facility frequently, in alignment with leadership expectations and the needs of the role. You may also be required to work from or visit a customer facility.&lt;/li&gt;&lt;li&gt;Onsite: If this position is listed as onsite, work will primarily be performed at a Booz Allen office or customer facility, where employees will collaborate directly with colleagues and customers as required by the role.&lt;br&gt;&lt;br&gt;&lt;br&gt;&lt;/li&gt;&lt;/ul&gt;&lt;strong&gt;Commitment to Non-Discrimination&lt;br&gt;&lt;br&gt;&lt;/strong&gt;All qualified applicants will receive consideration for employment without regard to disability, status as a protected veteran or any other status protected by applicable federal, state, local, or international law.</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Job Number: R0246928
+AI Developer
+The Opportunity: 
+As an experienced AI engineer, you know that AI systems are critical to understanding and processing massive datasets in an organization. Your ability to conduct statistical analyses on business processes using ML techniques makes you an integral part of delivering a customer-focused solution. We need your technical knowledge and desire to solve problems to support optimizing organizational efficiency. As an AI Developer on our Air Power team, you’ll train, test, deploy, and maintain models that learn from data.
+In this role, you’ll own and define the direction of mission-critical solutions by applying cutting-edge Agentic frameworks. You’ll be part of a large community of AI professionals across the company and collaborate with data engineers, data scientists, solutions architects, and product owners to deliver world-class solutions to transform how the Air Force manages its day-to-day business. Your skills and extensive technical expertise will guide clients as they navigate the landscape of Agentic Frameworks.
+Join us. The world can’t wait.
+You Have:
+- 2+ years of experience building production-grade software in Python, TypeScript, or Java with APIs and data services, including FastAPI, Flask, REST, GraphQL, or SQL
+- Experience developing and deploying AI-enabled applications such as LLMs, RAG, and agentic workflows to solve mission problems
+- Ability to design event-driven integrations and workflow automation such as asynchronous messaging or audit logging to move from insight to action
+- Ability to implement MLOps or DevSecOps practices such as CI/CD, containerization, automated testing, or model evaluation
+- Secret clearance
+- Bachelor’s degree in Mathematics, Computer Science, Software Engineering, or Data Science
+Nice If You Have:
+- Experience working with geospatial or 3D data, including point clouds, LiDAR, or photogrammetry, or digital-twin or facility and asset data models
+- Experience integrating sensor streams or IoT telemetry and edge-to-cloud data flows such as Kafka, NATS, RabbitMQ, or equivalent for asset monitoring and situational awareness
+- Experience deploying software and data or ML pipelines in disconnected, air-gapped, or classified environments
+- Experience with cross-domain data handling constraints
+- Experience with RMF or STIG-aligned delivery
+- Experience with AI-assisted software development tools and practices such as code copilots, automated tests, or secure-by-design patterns to increase delivery velocity responsibly
+- TS/SCI clearance
+Clearance: 
+Applicants selected will be subject to a security investigation and may need to meet eligibility requirements for access to classified information; Secret clearance is required.
+Compensation
+At Booz Allen, we celebrate your contributions, provide you with opportunities and choices, and support your total well-being. Our offerings include health, life, disability, financial, and retirement benefits, as well as paid leave, professional development, tuition assistance, work-life programs, and dependent care. Our recognition awards program acknowledges employees for exceptional performance and superior demonstration of our values. Full-time and part-time employees working at least 20 hours a week on a regular basis are eligible to participate in Booz Allen’s benefit programs. Individuals that do not meet the threshold are only eligible for select offerings, not inclusive of health benefits. We encourage you to learn more about our total benefits by visiting the Resource page on our Careers site and reviewing Our Employee Benefits page.
+Salary at Booz Allen is determined by various factors, including but not limited to location, the individual’s particular combination of education, knowledge, skills, competencies, and experience, as well as contract-specific affordability and organizational requirements. The projected compensation range for this position is $77,500.00 to $176,000.00 (annualized USD). The estimate displayed represents the typical salary range for this position and is just one component of Booz Allen’s total compensation package for employees. This posting will close within 90 days from the Posting Date.
+Identity Statement
+As part of the hiring process, we will ask you to complete an identity verification process that leverages advanced biometrics and artificial intelligence to ensure authenticity and protect against identity fraud. You are expected to be on camera during interviews and assessments. We reserve the right to take your picture to verify your identity and prevent fraud.
+Candidate AI Usage Policy
+AI is a part of our daily work at Booz Allen, and we are committed to the responsible and ethical use of AI tools. However, we want to ensure a fair candidate process based on your own skills and knowledge. As part of this commitment, the use of artificial intelligence (AI) or other tools to assist with responses during interviews (whether in-person or virtual) is prohibited unless permission is explicitly provided.
+Work Model
+Our people-first culture prioritizes the benefits of collaboration, whether it occurs in person or virtually. To support engagement and effective communication, employees working virtually are generally expected to have their cameras on during meetings.
+- Remote: If this position is listed as remote, there may still be occasions when you are required to work in person at a Booz Allen or customer facility.
+- Hybrid: If this position is listed as hybrid, you will be expected to work from a Booz Allen facility frequently, in alignment with leadership expectations and the needs of the role. You may also be required to work from or visit a customer facility.
+- Onsite: If this position is listed as onsite, work will primarily be performed at a Booz Allen office or customer facility, where employees will collaborate directly with colleagues and customers as required by the role.
+Commitment to Non-Discrimination
+All qualified applicants will receive consideration for employment without regard to disability, status as a protected veteran or any other status protected by applicable federal, state, local, or international law.</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Engineering and Information Technology</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Software Development</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?position=1&amp;pageNum=0&amp;keywords=AI+Engineer&amp;location=United+States&amp;distance=0&amp;f_TPR=r86400</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>{'type': 'PostalAddress', 'streetAddress': '8283 Greensboro Drive', 'addressLocality': 'McLean', 'addressRegion': 'VA', 'postalCode': '22102', 'addressCountry': 'US'}</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>https://boozallen.co/3PbO3a2</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr"/>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Whether at the border, up in space, or on the battlefield, we build the advanced technology that makes America stronger, faster, and safer. It’s who we are and what we do. It’s in our code. </t>
+        </is>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>37257</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>2026-08-14 05:10:51</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr"/>
+      <c r="AD24" t="inlineStr"/>
+      <c r="AE24" t="inlineStr"/>
+      <c r="AF24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>4426733766</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>XQYJD1Wcn8a5HPS6YzIHtg==</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Hqan1SC6SBVwlDMjIWeHxQ==</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/agentic-ai-engineer-%E2%80%94-healthcare-ai-at-deloitte-4426733766?position=10&amp;pageNum=0&amp;refId=Hqan1SC6SBVwlDMjIWeHxQ%3D%3D&amp;trackingId=XQYJD1Wcn8a5HPS6YzIHtg%3D%3D</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Agentic AI Engineer — Healthcare AI</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Deloitte</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/deloitte?trk=public_jobs_jserp-result_job-search-card-subtitle</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>https://media.licdn.com/dms/image/v2/C560BAQGNtpblgQpJoQ/company-logo_100_100/company-logo_100_100/0/1662120928214/deloitte_logo?e=2147483647&amp;v=beta&amp;t=OSF8M5LreT0Sf2F-JcNk6XMT0ArCuPfDmRR-knCC4HY</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>San Jose, CA</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Three hundred fifty million Americans rely on a healthcare system whose decision-making has become slow, costly, and adversarial - care delayed by prior authorization and paperwork, claims that misfire, clinical decisions made without the right information at the right moment, and patients who struggle to navigate or afford the care they need. Deloitte has a new AI-first effort, backed by $1B in committed investment, building the reasoning models and agentic systems to rebuild how that system decides - across payers, providers, and life sciences, and for the patients they serve - so that care is faster, fairer, and far less wasteful. This is not AI applied at the margins. It is a ground-up rebuild of the decision-making machinery behind American healthcare, at national scale.&lt;br&gt;&lt;br&gt;This is an early, well-funded build. You will own agent systems end to end - from architecture through production - and your work ships into live clinical and operational settings within your first months, not into a lab.&lt;br&gt;&lt;br&gt;As an Agentic AI Engineer, you will design, build, and operationalize the LLM- and SLM-powered systems behind real healthcare decisioning - the reasoning, orchestration, retrieval, memory, and control layers that let intelligent agents operate reliably across the hardest decisions in the industry: clinical reasoning, prior authorization and claims integrity, care navigation, and the operational workflows that run across payers, providers, and life sciences. This is not a prompt-only role. We are looking for builders who think deeply about system behavior, grounding, and reliability where a wrong action has real consequences for patients and the clinicians who serve them.&lt;br&gt;&lt;br&gt;You do not need a healthcare background. We pair every engineer with clinical and domain experts and teach you the domain - you bring the agentic engineering depth.&lt;br&gt;&lt;br&gt;We hire on demonstrated depth, not years - the level you join at is determined through our interview process, based on the depth and judgment you demonstrate, not your years in a title.&lt;br&gt;&lt;br&gt;Work you'll do&lt;br&gt;&lt;br&gt;Agent architecture &amp;amp; orchestration&lt;br&gt;&lt;br&gt;&lt;ul&gt;&lt;li&gt; Design and implement agentic systems capable of multi-step reasoning, planning, tool use, and workflow execution against complex, regulated operational processes.&lt;/li&gt;&lt;li&gt; Build stateful workflows using frameworks such as LangGraph and LangChain - including branching, retries, self-correction, human-in-the-loop checkpoints, and reusable orchestration patterns.&lt;/li&gt;&lt;li&gt; Engineer for long-horizon reliability - multi-step task completion, recovery from compounding errors, planning under uncertainty, and robust tool use when individual steps fail.&lt;/li&gt;&lt;li&gt; Build the reasoning behind regulated decisions - policy- and criteria-grounded outputs, structured proposer/critic/judge-style review, and auditable rationales for high-stakes decisions across the industry, from clinical review and prior authorization to claims integrity and care management.&lt;br&gt;&lt;br&gt;&lt;/li&gt;&lt;/ul&gt;Retrieval, grounding &amp;amp; context engineering&lt;br&gt;&lt;br&gt;&lt;ul&gt;&lt;li&gt; Develop end-to-end Retrieval-Augmented Generation (RAG) pipelines: ingestion, chunking, embeddings, vector and hybrid retrieval, reranking, contextual compression, and grounding strategies.&lt;/li&gt;&lt;li&gt; Engineer memory and context management - conversational state, persistent memory, retrieval-aware context assembly, and token-efficient context selection.&lt;/li&gt;&lt;li&gt; Apply modern context-delivery patterns (e.g., MCP-style tool/context interfaces) so agents access the right information at the right time.&lt;br&gt;&lt;br&gt;&lt;/li&gt;&lt;/ul&gt;Reliability, evaluation &amp;amp; safety&lt;br&gt;&lt;br&gt;&lt;ul&gt;&lt;li&gt; Implement observability and tracing for prompts, tool calls, retrieval quality, agent traces, failures, drift, latency, and production behavior.&lt;/li&gt;&lt;li&gt; Apply guardrails, safety controls, and failure-handling to reduce hallucinations and unsafe actions.&lt;/li&gt;&lt;li&gt; Evaluate agents at the trajectory and task level - multi-step task success, failure-mode and regression analysis, and sandboxed test environments - alongside retrieval- and generation-quality metrics, automated checks, and human review.&lt;/li&gt;&lt;li&gt; Engineer healthcare-grade safety - deployment eval gates, human-oversight and escalation models, auditability and traceability for regulated decisions, and PHI/HIPAA-aware data handling.&lt;br&gt;&lt;br&gt;&lt;/li&gt;&lt;/ul&gt;Integration &amp;amp; production craft&lt;br&gt;&lt;br&gt;&lt;ul&gt;&lt;li&gt; Build integrations with internal and external tools, APIs, enterprise systems, databases, and model providers so agents operate safely within real business workflows.&lt;/li&gt;&lt;li&gt; Deliver production-quality code with strong practices in testing, CI/CD, logging, versioning, and documentation; make architecture decisions that balance quality, safety, latency, cost, and model risk.&lt;/li&gt;&lt;li&gt; Partner with our modeling and post-training engineers to improve model behavior for tool use, grounding, and long-horizon reasoning - through evaluation-driven feedback and, where it helps, fine-tuned or reasoning-optimized models.&lt;/li&gt;&lt;li&gt; Translate ambiguous, high-complexity operational processes into robust system logic and reusable AI patterns; stay current with advances in agentic systems and translate research into practical engineering decisions.&lt;br&gt;&lt;br&gt;&lt;/li&gt;&lt;/ul&gt;The team&lt;br&gt;&lt;br&gt;Deloitte brings together AI researchers, modeling and platform engineers, architects, clinical and domain specialists, and product leaders to build, deploy, and operate verticalized AI systems across software, data, models, and cloud infrastructure - engineered for one of the most complex operating environments in the world. The work spans the healthcare industry - payers, providers, and life sciences - and involves genuinely hard reasoning problems, nuanced operational workflows, and a high bar for reliability, with little tolerance for shallow or unreliable outputs. We pair frontier AI research with production-grade engineering, and we ship into real clinical and operational settings rather than leaving models in the lab.&lt;br&gt;&lt;br&gt;&lt;strong&gt;Required Qualifications&lt;br&gt;&lt;br&gt;&lt;/strong&gt;&lt;ul&gt;&lt;li&gt; Bachelor's degree in Computer Science, Engineering, Data Science, Computational Linguistics, or a related field.&lt;/li&gt;&lt;li&gt; Demonstrated depth building and shipping production agentic systems - this is your primary craft, not a recent exploration. We weigh shipped systems, research, model releases, and open source over years in a title; expect strong software/ML fundamentals plus substantial, recent hands-on agentic work.&lt;/li&gt;&lt;li&gt; Strong, hands-on experience building production agent systems with modern orchestration - LangGraph/LangChain or equivalent, including custom orchestration.&lt;/li&gt;&lt;li&gt; Experience designing and optimizing end-to-end RAG systems: indexing, retrieval, reranking, grounding, and evaluation.&lt;/li&gt;&lt;li&gt; Strong understanding of memory and context management, including context windows, retrieval-driven context assembly, persistent memory, and high-signal context selection.&lt;/li&gt;&lt;li&gt; Deep, practical understanding of LLM behavior - strengths, limitations, hallucination risks, reasoning constraints, and latency/cost trade-offs - and the evaluation methods used to measure them.&lt;/li&gt;&lt;li&gt; Experience evaluating and debugging agent behavior - task-success and trajectory analysis, not just output quality.&lt;/li&gt;&lt;li&gt; Strong Python engineering skills and modern software practices: testing, CI/CD, version control, and API integration; experience implementing observability, tracing, and debugging for LLM-based systems in production.&lt;/li&gt;&lt;li&gt; Hands-on experience with at least one frontier model platform (e.g., Anthropic, Google, OpenAI) and/or open-weight/self-hosted models (e.g., Llama via vLLM), including production tool use and agent capabilities.&lt;/li&gt;&lt;li&gt; Ability to travel 0-50%, on average, based on the work you do and the clients and industries/sectors you serve.&lt;/li&gt;&lt;li&gt; Limited immigration sponsorship may be available.&lt;br&gt;&lt;br&gt;&lt;/li&gt;&lt;/ul&gt;&lt;strong&gt;Preferred Qualifications&lt;br&gt;&lt;br&gt;&lt;/strong&gt;&lt;ul&gt;&lt;li&gt; Experience with multi-agent systems and agent collaboration patterns.&lt;/li&gt;&lt;li&gt; Familiarity with vector databases and retrieval infrastructure such as Pinecone, Weaviate, or Milvus.&lt;/li&gt;&lt;li&gt; Exposure to model adaptation and fine-tuning techniques such as LoRA or QLoRA.&lt;/li&gt;&lt;li&gt; Understanding of traditional NLP concepts: tokenization, semantic similarity, entity extraction, summarization, and transformer fundamentals.&lt;/li&gt;&lt;li&gt; Experience operating in highly regulated, high-stakes, or operationally complex environments; healthcare exposure - clinical, payer, or life-sciences workflows, or standards such as FHIR - is a plus, not a requirement.&lt;/li&gt;&lt;li&gt; Demonstrated habit of staying current with AI research, benchmarks, and emerging engineering patterns.&lt;br&gt;&lt;br&gt;&lt;/li&gt;&lt;/ul&gt;&lt;strong&gt;Compensation&lt;br&gt;&lt;br&gt;&lt;/strong&gt;Base salary is benchmarked to leading technology companies rather than traditional consulting scales, and the role carries a substantial performance-based incentive opportunity designed to grow with the value you help create - startup-style upside, with the backing of a committed, well-capitalized platform. The estimated base salary range is $110,700-$372,900 (not adjusted for geographic differential); actual base pay depends on your skills, experience, and level, and you may also be eligible for a discretionary annual incentive based on individual and organizational performance.</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>163</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Three hundred fifty million Americans rely on a healthcare system whose decision-making has become slow, costly, and adversarial - care delayed by prior authorization and paperwork, claims that misfire, clinical decisions made without the right information at the right moment, and patients who struggle to navigate or afford the care they need. Deloitte has a new AI-first effort, backed by $1B in committed investment, building the reasoning models and agentic systems to rebuild how that system decides - across payers, providers, and life sciences, and for the patients they serve - so that care is faster, fairer, and far less wasteful. This is not AI applied at the margins. It is a ground-up rebuild of the decision-making machinery behind American healthcare, at national scale.
+This is an early, well-funded build. You will own agent systems end to end - from architecture through production - and your work ships into live clinical and operational settings within your first months, not into a lab.
+As an Agentic AI Engineer, you will design, build, and operationalize the LLM- and SLM-powered systems behind real healthcare decisioning - the reasoning, orchestration, retrieval, memory, and control layers that let intelligent agents operate reliably across the hardest decisions in the industry: clinical reasoning, prior authorization and claims integrity, care navigation, and the operational workflows that run across payers, providers, and life sciences. This is not a prompt-only role. We are looking for builders who think deeply about system behavior, grounding, and reliability where a wrong action has real consequences for patients and the clinicians who serve them.
+You do not need a healthcare background. We pair every engineer with clinical and domain experts and teach you the domain - you bring the agentic engineering depth.
+We hire on demonstrated depth, not years - the level you join at is determined through our interview process, based on the depth and judgment you demonstrate, not your years in a title.
+Work you'll do
+Agent architecture &amp;amp; orchestration
+-  Design and implement agentic systems capable of multi-step reasoning, planning, tool use, and workflow execution against complex, regulated operational processes.
+-  Build stateful workflows using frameworks such as LangGraph and LangChain - including branching, retries, self-correction, human-in-the-loop checkpoints, and reusable orchestration patterns.
+-  Engineer for long-horizon reliability - multi-step task completion, recovery from compounding errors, planning under uncertainty, and robust tool use when individual steps fail.
+-  Build the reasoning behind regulated decisions - policy- and criteria-grounded outputs, structured proposer/critic/judge-style review, and auditable rationales for high-stakes decisions across the industry, from clinical review and prior authorization to claims integrity and care management.
+Retrieval, grounding &amp;amp; context engineering
+-  Develop end-to-end Retrieval-Augmented Generation (RAG) pipelines: ingestion, chunking, embeddings, vector and hybrid retrieval, reranking, contextual compression, and grounding strategies.
+-  Engineer memory and context management - conversational state, persistent memory, retrieval-aware context assembly, and token-efficient context selection.
+-  Apply modern context-delivery patterns (e.g., MCP-style tool/context interfaces) so agents access the right information at the right time.
+Reliability, evaluation &amp;amp; safety
+-  Implement observability and tracing for prompts, tool calls, retrieval quality, agent traces, failures, drift, latency, and production behavior.
+-  Apply guardrails, safety controls, and failure-handling to reduce hallucinations and unsafe actions.
+-  Evaluate agents at the trajectory and task level - multi-step task success, failure-mode and regression analysis, and sandboxed test environments - alongside retrieval- and generation-quality metrics, automated checks, and human review.
+-  Engineer healthcare-grade safety - deployment eval gates, human-oversight and escalation models, auditability and traceability for regulated decisions, and PHI/HIPAA-aware data handling.
+Integration &amp;amp; production craft
+-  Build integrations with internal and external tools, APIs, enterprise systems, databases, and model providers so agents operate safely within real business workflows.
+-  Deliver production-quality code with strong practices in testing, CI/CD, logging, versioning, and documentation; make architecture decisions that balance quality, safety, latency, cost, and model risk.
+-  Partner with our modeling and post-training engineers to improve model behavior for tool use, grounding, and long-horizon reasoning - through evaluation-driven feedback and, where it helps, fine-tuned or reasoning-optimized models.
+-  Translate ambiguous, high-complexity operational processes into robust system logic and reusable AI patterns; stay current with advances in agentic systems and translate research into practical engineering decisions.
+The team
+Deloitte brings together AI researchers, modeling and platform engineers, architects, clinical and domain specialists, and product leaders to build, deploy, and operate verticalized AI systems across software, data, models, and cloud infrastructure - engineered for one of the most complex operating environments in the world. The work spans the healthcare industry - payers, providers, and life sciences - and involves genuinely hard reasoning problems, nuanced operational workflows, and a high bar for reliability, with little tolerance for shallow or unreliable outputs. We pair frontier AI research with production-grade engineering, and we ship into real clinical and operational settings rather than leaving models in the lab.
+Required Qualifications
+-  Bachelor's degree in Computer Science, Engineering, Data Science, Computational Linguistics, or a related field.
+-  Demonstrated depth building and shipping production agentic systems - this is your primary craft, not a recent exploration. We weigh shipped systems, research, model releases, and open source over years in a title; expect strong software/ML fundamentals plus substantial, recent hands-on agentic work.
+-  Strong, hands-on experience building production agent systems with modern orchestration - LangGraph/LangChain or equivalent, including custom orchestration.
+-  Experience designing and optimizing end-to-end RAG systems: indexing, retrieval, reranking, grounding, and evaluation.
+-  Strong understanding of memory and context management, including context windows, retrieval-driven context assembly, persistent memory, and high-signal context selection.
+-  Deep, practical understanding of LLM behavior - strengths, limitations, hallucination risks, reasoning constraints, and latency/cost trade-offs - and the evaluation methods used to measure them.
+-  Experience evaluating and debugging agent behavior - task-success and trajectory analysis, not just output quality.
+-  Strong Python engineering skills and modern software practices: testing, CI/CD, version control, and API integration; experience implementing observability, tracing, and debugging for LLM-based systems in production.
+-  Hands-on experience with at least one frontier model platform (e.g., Anthropic, Google, OpenAI) and/or open-weight/self-hosted models (e.g., Llama via vLLM), including production tool use and agent capabilities.
+-  Ability to travel 0-50%, on average, based on the work you do and the clients and industries/sectors you serve.
+-  Limited immigration sponsorship may be available.
+Preferred Qualifications
+-  Experience with multi-agent systems and agent collaboration patterns.
+-  Familiarity with vector databases and retrieval infrastructure such as Pinecone, Weaviate, or Milvus.
+-  Exposure to model adaptation and fine-tuning techniques such as LoRA or QLoRA.
+-  Understanding of traditional NLP concepts: tokenization, semantic similarity, entity extraction, summarization, and transformer fundamentals.
+-  Experience operating in highly regulated, high-stakes, or operationally complex environments; healthcare exposure - clinical, payer, or life-sciences workflows, or standards such as FHIR - is a plus, not a requirement.
+-  Demonstrated habit of staying current with AI research, benchmarks, and emerging engineering patterns.
+Compensation
+Base salary is benchmarked to leading technology companies rather than traditional consulting scales, and the role carries a substantial performance-based incentive opportunity designed to grow with the value you help create - startup-style upside, with the backing of a committed, well-capitalized platform. The estimated base salary range is $110,700-$372,900 (not adjusted for geographic differential); actual base pay depends on your skills, experience, and level, and you may also be eligible for a discretionary annual incentive based on individual and organizational performance.</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Engineering and Information Technology</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>Accounting, IT Services and IT Consulting, and Business Consulting and Services</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?position=1&amp;pageNum=0&amp;keywords=AI+Engineer&amp;location=United+States&amp;distance=0&amp;f_TPR=r86400</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>{'type': 'PostalAddress', 'streetAddress': 'Worldwide', 'addressLocality': 'Worldwide', 'addressCountry': 'OO'}</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>http://www.deloitte.com/</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>Together makes progress</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>Deloitte drives progress. Our firms around the world help clients become leaders wherever they choose to compete. Deloitte invests in outstanding people of diverse talents and backgrounds and empowers them to achieve more than they could elsewhere. Our work combines advice with action and integrity. We believe that when our clients and society are stronger, so are we. 
+Deloitte refers to one or more of Deloitte Touche Tohmatsu Limited (“DTTL”), its global network of member firms, and their related entities. DTTL (also referred to as “Deloitte Global”) and each of its member firms are legally separate and independent entities. DTTL does not provide services to clients. Please see www.deloitte.com/about to learn more.
+The content on this page contains general information only, and none of Deloitte Touche Tohmatsu Limited, its member firms, or their related entities (collectively the “Deloitte Network”) is, by means of this publication, rendering professional advice or services. Before making any decision or taking any action that may affect your finances or your business, you should consult a qualified professional adviser. No entity in the Deloitte Network shall be responsible for any loss whatsoever sustained by any person who relies on content from this page.</t>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>532502</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>2026-08-14 05:10:51</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr"/>
+      <c r="AD25" t="inlineStr"/>
+      <c r="AE25" t="inlineStr"/>
+      <c r="AF25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>4453270200</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Ff5GK9IMT2kdjYzk9ubFug==</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Hqan1SC6SBVwlDMjIWeHxQ==</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-tata-consultancy-services-4453270200?position=6&amp;pageNum=0&amp;refId=Hqan1SC6SBVwlDMjIWeHxQ%3D%3D&amp;trackingId=Ff5GK9IMT2kdjYzk9ubFug%3D%3D</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>AI/ML Engineer</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/company/tata-consultancy-services?trk=public_jobs_jserp-result_job-search-card-subtitle</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>https://media.licdn.com/dms/image/v2/D4D0BAQGsGR9p4ikS5w/company-logo_100_100/company-logo_100_100/0/1708946550425/tata_consultancy_services_logo?e=2147483647&amp;v=beta&amp;t=P-PkUMh7Ks1GQY0_l7GhzQiwfyLfQpvKWwX8Tq18Yc4</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Los Angeles, CA</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>&lt;strong&gt;Job Description&lt;br&gt;&lt;br&gt;&lt;/strong&gt;Must Have Technical/Functional Skills&lt;br&gt;&lt;br&gt;&lt;ul&gt;&lt;li&gt; Python (Expert level)&lt;/li&gt;&lt;li&gt; Machine Learning &amp;amp; Model Training&lt;/li&gt;&lt;li&gt;Training, evaluation, fine tuning&lt;/li&gt;&lt;li&gt;Tagging and labeling workflows&lt;/li&gt;&lt;li&gt; Generative AI &amp;amp; LLMs&lt;/li&gt;&lt;li&gt;Prompt engineering for LLM-based applications&lt;/li&gt;&lt;li&gt; Document Processing&lt;/li&gt;&lt;li&gt;Document extraction, parsing, and chunking&lt;/li&gt;&lt;li&gt;Handling structured &amp;amp; unstructured data&lt;/li&gt;&lt;li&gt; Embeddings &amp;amp; Vector Search&lt;/li&gt;&lt;li&gt;Embedding generation&lt;/li&gt;&lt;li&gt;Vector database integration&lt;/li&gt;&lt;li&gt; Databases&lt;/li&gt;&lt;li&gt;Vector Databases&lt;/li&gt;&lt;li&gt;MongoDB&lt;/li&gt;&lt;li&gt; Production-grade ML Engineering&lt;/li&gt;&lt;li&gt;Scalable, production-ready ML/GenAI solutions&lt;br&gt;&lt;br&gt;&lt;/li&gt;&lt;/ul&gt;Roles &amp;amp; Responsibilities&lt;br&gt;&lt;br&gt;This role is for a hands-on AI/ML Engineer who will design, build, and deploy production‑grade Machine Learning and Generative AI solutions. The candidate must have strong Python expertise and practical experience taking ML and GenAI use cases from development to deployment.&lt;br&gt;&lt;br&gt;The role focuses heavily on LLM-based applications, including prompt engineering, document processing pipelines, and embedding-based search solutions. The engineer will work with both structured and unstructured data, building pipelines for document extraction, parsing, and chunking, and integrating ML models with Vector Databases and MongoDB.&lt;br&gt;&lt;br&gt;An ideal candidate is someone who understands end-to-end ML workflows—from data preparation, tagging, and labeling, through model training, evaluation, and fine-tuning—while ensuring solutions are scalable, high quality, and production ready.&lt;br&gt;&lt;br&gt;For recruiter to interpret accurately&lt;br&gt;&lt;br&gt;&lt;ul&gt;&lt;li&gt; Not a pure data analyst → this is an engineering-focused ML/GenAI role&lt;/li&gt;&lt;li&gt; Not theoretical AI → requires real-world deployment experience&lt;/li&gt;&lt;li&gt; Strong fit for candidates with backgrounds in:&lt;/li&gt;&lt;li&gt;ML Engineering&lt;/li&gt;&lt;li&gt;Applied Data Science&lt;/li&gt;&lt;li&gt;GenAI / LLM application development&lt;br&gt;&lt;br&gt;&lt;/li&gt;&lt;/ul&gt;Key Responsibilities&lt;br&gt;&lt;br&gt;&lt;ul&gt;&lt;li&gt; Design and implement AI/ML solutions using Python and modern ML frameworks&lt;/li&gt;&lt;li&gt; Develop and optimize Prompt Engineering strategies for LLM-based systems&lt;/li&gt;&lt;li&gt; Build and deploy Retrieval-Augmented Generation (RAG) pipelines&lt;/li&gt;&lt;li&gt; Integrate LLMs via APIs (Azure OpenAI preferred) into enterprise applications&lt;/li&gt;&lt;li&gt; Develop and orchestrate Agent ic AI workflows with tool/function calling&lt;/li&gt;&lt;li&gt; Implement vector search solutions using Vector Databases&lt;/li&gt;&lt;li&gt; Ensure CI/CD integration and cloud deployment (Azure preferred)&lt;/li&gt;&lt;li&gt; Establish observability, monitoring, and evaluation frameworks for AI systems&lt;/li&gt;&lt;li&gt; Collaborate with cross-functional teams to deliver production-ready AI features&lt;br&gt;&lt;br&gt;&lt;/li&gt;&lt;/ul&gt;Generic Managerial Skills, If any&lt;br&gt;&lt;br&gt;&lt;ul&gt;&lt;li&gt; Ability to explain complex ML / GenAI concepts to non‑technical stakeholders and collaborate effectively with cross‑functional teams.&lt;/li&gt;&lt;li&gt; Strong analytical thinking to break down ambiguous business problems into workable ML or GenAI solutions.&lt;/li&gt;&lt;li&gt; Takes end‑to‑end responsibility for solutions—from design to production readiness—without constant supervision.&lt;/li&gt;&lt;li&gt; Works well with data engineers, product owners, and platform teams to deliver integrated, scalable solutions.&lt;/li&gt;&lt;li&gt; Actively keeps up with evolving ML, LLM, and GenAI technologies and improves skills proactively.&lt;br&gt;&lt;br&gt;&lt;/li&gt;&lt;/ul&gt;Salary Range: $140,000 -$165,000 year&lt;br&gt;&lt;br&gt;&lt;strong&gt;TCS Employee Benefits Summary&lt;br&gt;&lt;br&gt;&lt;/strong&gt;Discretionary Annual Incentive.&lt;br&gt;&lt;br&gt;Comprehensive Medical Coverage: Medical &amp;amp; Health, Dental &amp;amp; Vision, Disability Planning &amp;amp; Insurance, Pet Insurance Plans.&lt;br&gt;&lt;br&gt;Family Support: Maternal &amp;amp; Parental Leaves.&lt;br&gt;&lt;br&gt;Insurance Options: Auto &amp;amp; Home Insurance, Identity Theft Protection.&lt;br&gt;&lt;br&gt;Convenience &amp;amp; Professional Growth: Commuter Benefits &amp; Certification &amp; amp; Training Reimbursement.&lt;br&gt;&lt;br&gt;Time Off: Vacation, Time Off, Sick Leave &amp;amp; Holidays.&lt;br&gt;&lt;br&gt;Legal &amp;amp; Financial Assistance: Legal Assistance, 401K Plan, Performance Bonus, College Fund, Student Loan Refinancing.&lt;br&gt;&lt;br&gt;&lt;strong&gt;Qualifications: &lt;/strong&gt;BACHELOR OF COMPUTER SCIENCE&lt;br&gt;&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Job Description
+Must Have Technical/Functional Skills
+-  Python (Expert level)
+-  Machine Learning &amp;amp; Model Training
+- Training, evaluation, fine tuning
+- Tagging and labeling workflows
+-  Generative AI &amp;amp; LLMs
+- Prompt engineering for LLM-based applications
+-  Document Processing
+- Document extraction, parsing, and chunking
+- Handling structured &amp;amp; unstructured data
+-  Embeddings &amp;amp; Vector Search
+- Embedding generation
+- Vector database integration
+-  Databases
+- Vector Databases
+- MongoDB
+-  Production-grade ML Engineering
+- Scalable, production-ready ML/GenAI solutions
+Roles &amp;amp; Responsibilities
+This role is for a hands-on AI/ML Engineer who will design, build, and deploy production‑grade Machine Learning and Generative AI solutions. The candidate must have strong Python expertise and practical experience taking ML and GenAI use cases from development to deployment.
+The role focuses heavily on LLM-based applications, including prompt engineering, document processing pipelines, and embedding-based search solutions. The engineer will work with both structured and unstructured data, building pipelines for document extraction, parsing, and chunking, and integrating ML models with Vector Databases and MongoDB.
+An ideal candidate is someone who understands end-to-end ML workflows—from data preparation, tagging, and labeling, through model training, evaluation, and fine-tuning—while ensuring solutions are scalable, high quality, and production ready.
+For recruiter to interpret accurately
+-  Not a pure data analyst → this is an engineering-focused ML/GenAI role
+-  Not theoretical AI → requires real-world deployment experience
+-  Strong fit for candidates with backgrounds in:
+- ML Engineering
+- Applied Data Science
+- GenAI / LLM application development
+Key Responsibilities
+-  Design and implement AI/ML solutions using Python and modern ML frameworks
+-  Develop and optimize Prompt Engineering strategies for LLM-based systems
+-  Build and deploy Retrieval-Augmented Generation (RAG) pipelines
+-  Integrate LLMs via APIs (Azure OpenAI preferred) into enterprise applications
+-  Develop and orchestrate Agent ic AI workflows with tool/function calling
+-  Implement vector search solutions using Vector Databases
+-  Ensure CI/CD integration and cloud deployment (Azure preferred)
+-  Establish observability, monitoring, and evaluation frameworks for AI systems
+-  Collaborate with cross-functional teams to deliver production-ready AI features
+Generic Managerial Skills, If any
+-  Ability to explain complex ML / GenAI concepts to non‑technical stakeholders and collaborate effectively with cross‑functional teams.
+-  Strong analytical thinking to break down ambiguous business problems into workable ML or GenAI solutions.
+-  Takes end‑to‑end responsibility for solutions—from design to production readiness—without constant supervision.
+-  Works well with data engineers, product owners, and platform teams to deliver integrated, scalable solutions.
+-  Actively keeps up with evolving ML, LLM, and GenAI technologies and improves skills proactively.
+Salary Range: $140,000 -$165,000 year
+TCS Employee Benefits Summary
+Discretionary Annual Incentive.
+Comprehensive Medical Coverage: Medical &amp;amp; Health, Dental &amp;amp; Vision, Disability Planning &amp;amp; Insurance, Pet Insurance Plans.
+Family Support: Maternal &amp;amp; Parental Leaves.
+Insurance Options: Auto &amp;amp; Home Insurance, Identity Theft Protection.
+Convenience &amp;amp; Professional Growth: Commuter Benefits &amp; Certification &amp; amp; Training Reimbursement.
+Time Off: Vacation, Time Off, Sick Leave &amp;amp; Holidays.
+Legal &amp;amp; Financial Assistance: Legal Assistance, 401K Plan, Performance Bonus, College Fund, Student Loan Refinancing.
+Qualifications: BACHELOR OF COMPUTER SCIENCE
+</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>Engineering and Information Technology</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>IT Services and IT Consulting</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?position=1&amp;pageNum=0&amp;keywords=AI+Engineer&amp;location=United+States&amp;distance=0&amp;f_TPR=r86400</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>{'type': 'PostalAddress', 'streetAddress': 'Tata Consultancy Services', 'addressLocality': 'Mumbai', 'addressRegion': 'Maharashtra', 'postalCode': '400001', 'addressCountry': 'IN'}</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>https://www.tcs.com/</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services (TCS) is the technology partner of choice for industry leading organizations worldwide. Since its inception in 1968, TCS has upheld the highest standards of innovation, engineering excellence, and customer service. 
+It has set an aspiration to become the world's largest AI-led technology services company and is enabling its clients to transform themselves across the full AI stack, from infrastructure to intelligence. 
+Rooted in the heritage of the Tata Group, TCS is focused on creating long term value for its clients, its investors, its employees, and the community at large. With a highly skilled workforce spread across 55 countries and 202 service delivery centers across the world, the company has been recognized as a top employer in six continents. With the ability to rapidly apply and scale new technologies, the company has built long term partnerships with its clients – helping them emerge as perpetually adaptive enterprises. Many of these relationships have endured into decades and navigated every technology cycle, from mainframes in the 1970s to artificial intelligence today. 
+TCS sponsors 14 of the world’s most prestigious marathons and endurance events, including the TCS New York City Marathon, TCS London Marathon and TCS Sydney Marathon with a focus on promoting health, sustainability, and community empowerment. 
+Caution against fraudulent job offers: TCS doesn’t charge any fee throughout the recruitment process. Refer here: https://www.tcs.com/careers/india/recruitment-fraud-alert</t>
+        </is>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>724977</t>
+        </is>
+      </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>2026-08-14 05:10:51</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr"/>
+      <c r="AD26" t="inlineStr"/>
+      <c r="AE26" t="inlineStr"/>
+      <c r="AF26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>4454057834</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>4BwzntIQuBpekghj0K1opA==</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Hqan1SC6SBVwlDMjIWeHxQ==</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-harnham-4454057834?position=5&amp;pageNum=0&amp;refId=Hqan1SC6SBVwlDMjIWeHxQ%3D%3D&amp;trackingId=4BwzntIQuBpekghj0K1opA%3D%3D</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>AI/ML Engineer</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Harnham</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>https://uk.linkedin.com/company/harnham?trk=public_jobs_jserp-result_job-search-card-subtitle</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>https://media.licdn.com/dms/image/v2/D4E0BAQFDh4hZFsU8qA/company-logo_100_100/company-logo_100_100/0/1732180104917/harnham_logo?e=2147483647&amp;v=beta&amp;t=2K2PZUjKIx7QPtNOXOgU2XOjaiYyj1Gnd8g_8LaDJhc</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>San Francisco Bay Area</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Title&lt;/strong&gt;: AI/ML Engineer (All Levels)&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Location&lt;/strong&gt;: Bay Area (Hybrid)&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Compensation&lt;/strong&gt;: Up to $350,000 + Equity&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;We're partnered with a well-funded, high-growth Series B startup building the next generation of AI-native data infrastructure for Fortune 500 enterprises. With 3.5x revenue growth in FY'24 and 160% net revenue retention, they're scaling fast and investing heavily in the AI engineering team that powers their core product.&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;This is a high-impact role where you'll own the intelligence layer of the platform, making real architectural decisions around agent design, model selection, and evaluation strategy. Everything you build ships directly to customers; this is not a POC or internal tooling team.&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;&lt;strong&gt;What You'll Do&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Architect multi-step AI agents end-to-end, covering problem decomposition, context retrieval, error recovery, and output quality&lt;/li&gt;&lt;li&gt;Own RAG pipelines, vector and graph-based retrieval systems, and knowledge representations that let agents reason accurately over complex enterprise data&lt;/li&gt;&lt;li&gt;Build the AI layer behind the platform's core code generation capability, from prompt design and model selection through to fine-tuning and output validation&lt;/li&gt;&lt;li&gt;Make production AI work at scale, balancing latency, throughput, and observability, and knowing when to optimize a model versus restructure a system&lt;/li&gt;&lt;li&gt;Think in failure modes and evaluation strategy, not capability demos, and own the improvement loop&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Requirements&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;4-6+ years of software engineering experience with meaningful AI/ML depth&lt;/li&gt;&lt;li&gt;Proven experience building and shipping AI agents or coding agents in production&lt;/li&gt;&lt;li&gt;Strong Python skills with hands-on experience across RAG, vector databases, and knowledge graphs&lt;/li&gt;&lt;li&gt;Experience with LLM APIs, prompt engineering, fine-tuning, and structured outputs in production&lt;/li&gt;&lt;li&gt;Familiarity with AWS and Kubernetes for production AI deployment&lt;/li&gt;&lt;li&gt;Experience with data platforms such as Databricks, Snowflake, BigQuery, or Spark is a strong bonus&lt;/li&gt;&lt;li&gt;Scale or Go experience is a bonus&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;If you're a builder who thinks in failure modes, owns what you ship, and thrives in environments where last year's best practice is already obsolete, this is a rare opportunity to have direct leverage on a product used by some of the world's largest enterprises.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>166</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Title: AI/ML Engineer (All Levels)
+Location: Bay Area (Hybrid)
+Compensation: Up to $350,000 + Equity
+We're partnered with a well-funded, high-growth Series B startup building the next generation of AI-native data infrastructure for Fortune 500 enterprises. With 3.5x revenue growth in FY'24 and 160% net revenue retention, they're scaling fast and investing heavily in the AI engineering team that powers their core product.
+This is a high-impact role where you'll own the intelligence layer of the platform, making real architectural decisions around agent design, model selection, and evaluation strategy. Everything you build ships directly to customers; this is not a POC or internal tooling team.
+What You'll Do
+- Architect multi-step AI agents end-to-end, covering problem decomposition, context retrieval, error recovery, and output quality
+- Own RAG pipelines, vector and graph-based retrieval systems, and knowledge representations that let agents reason accurately over complex enterprise data
+- Build the AI layer behind the platform's core code generation capability, from prompt design and model selection through to fine-tuning and output validation
+- Make production AI work at scale, balancing latency, throughput, and observability, and knowing when to optimize a model versus restructure a system
+- Think in failure modes and evaluation strategy, not capability demos, and own the improvement loop
+Requirements
+- 4-6+ years of software engineering experience with meaningful AI/ML depth
+- Proven experience building and shipping AI agents or coding agents in production
+- Strong Python skills with hands-on experience across RAG, vector databases, and knowledge graphs
+- Experience with LLM APIs, prompt engineering, fine-tuning, and structured outputs in production
+- Familiarity with AWS and Kubernetes for production AI deployment
+- Experience with data platforms such as Databricks, Snowflake, BigQuery, or Spark is a strong bonus
+- Scale or Go experience is a bonus
+If you're a builder who thinks in failure modes, owns what you ship, and thrives in environments where last year's best practice is already obsolete, this is a rare opportunity to have direct leverage on a product used by some of the world's largest enterprises.</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>Software Development</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?position=1&amp;pageNum=0&amp;keywords=AI+Engineer&amp;location=United+States&amp;distance=0&amp;f_TPR=r86400</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>{'type': 'PostalAddress', 'streetAddress': 'Melbury House, 51 Wimbledon Hill Road', 'addressLocality': 'Wimbledon', 'addressRegion': 'London', 'postalCode': 'SW19 7QW', 'addressCountry': 'GB'}</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>http://www.harnham.com</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Harnham is the global leader in Data and AI talent solutions. </t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>Harnham provides specialist Data and AI recruitment and staffing services, along with bespoke training solutions, across multiple industry verticals, operating in the UK, the USA and EU - contact us today to discuss your requirements: info@harnham.com 
+Our recruitment and talent teams cover all aspects of the data and AI pipeline, from collection to consumption, across multiple data roles and functions. 
+Whether you need full-time staff, contract talent, specialized training, Data-qualified graduates, or C-suite executives, Harnham Group is equipped to fulfill all your data talent requirements.
+Our five core services:
+* ATD - Rockborne – our graduate development arm – deploys expertly trained data consultants, who have gone through an intensive 12-week data training programme. After two years in the scheme, your consultant could become a 
+* Contract / C2C / Freelance: Whether you're addressing a talent shortage, augmenting a project team, or encountering resource gaps, our specialist consultants offer bespoke interim talent solutions to address your unique challenges and drive success.
+* Full-Time / Direct Hiring: From early career professionals to senior management, our comprehensive services enable you to unearth outstanding data talent across various specializations, ensuring your organization thrives in the data-driven era.
+* Executive Search: With our dedicated executive search team and an extensive network encompassing the director to C-suite level, we assist both global corporations and ambitious startups in securing top-tier leadership talent to accomplish their goals.
+* GenAI, Prompt, LLM Training: Elevate your team's data expertise with our all-encompassing training programs covering essential tools and technologies such as Python, SQL, Machine Learning, LLM’s and AI. Highly bespoke, customised to your team learning requirements and budgets.</t>
+        </is>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>2026-08-14 05:10:51</t>
+        </is>
+      </c>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>George Ethell</t>
+        </is>
+      </c>
+      <c r="AD27" t="inlineStr">
+        <is>
+          <t>Helping Founders &amp; AI Leaders hire top Research, Machine Learning, and Software Engineering talent across World Models, AIGC, Multimodal AI, Agents…</t>
+        </is>
+      </c>
+      <c r="AE27" t="inlineStr">
+        <is>
+          <t>https://static.licdn.com/aero-v1/sc/h/9c8pery4andzj6ohjkjp54ma2</t>
+        </is>
+      </c>
+      <c r="AF27" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/georgeethell</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>4452934313</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>qoHAclyiBouGDbBgN98OcQ==</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Hqan1SC6SBVwlDMjIWeHxQ==</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/ai-engineer-llm-agentic-systems-at-auxo-talent-4452934313?position=4&amp;pageNum=0&amp;refId=Hqan1SC6SBVwlDMjIWeHxQ%3D%3D&amp;trackingId=qoHAclyiBouGDbBgN98OcQ%3D%3D</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>AI Engineer (LLM / Agentic Systems)</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Auxo Talent</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/auxotalent?trk=public_jobs_jserp-result_job-search-card-subtitle</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://media.licdn.com/dms/image/v2/D4D0BAQFd1BEyLRUXwg/company-logo_100_100/company-logo_100_100/0/1726121227211/auxotalent_logo?e=2147483647&amp;v=beta&amp;t=RgLpMT_wYZuTV1ghbvLv31T4i0TPZWmrHIIQEXVh1NI</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>San Francisco Bay Area</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;AI Engineer (LLM / Agentic Systems)&lt;/strong&gt;&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Bay Area, California | Hybrid | $140,000 to $160,000 + equity&lt;/strong&gt;&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;A well-funded early stage company is applying AI to the operational side of critical infrastructure. Their platform pulls live data from sensor and control networks across large facilities, then uses agentic AI to spot problems, connect related events and give operators recommendations in real time. It is a genuinely hard technical problem in a market that is growing quickly.&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;This suits an engineer with roughly three to six years behind them who has already shipped LLM-powered systems into production and wants more ownership than a large team allows. You would be joining a small engineering group and working end to end, from data pipelines and model integration through to agentic orchestration, evaluation and production support.&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;It is not a research role, but research thinking matters. You will be expected to keep up with the field, bring ideas forward and then build them properly.&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;&lt;strong&gt;What you will work on&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Multi-agent orchestration and LLM-driven triage workflows&lt;/li&gt;&lt;li&gt;Time-series modelling for anomaly detection and failure prediction on multivariate data&lt;/li&gt;&lt;li&gt;Retrieval-augmented knowledge systems for operations teams&lt;/li&gt;&lt;li&gt;Data and ML pipelines: ingestion, ETL and dataset construction&lt;/li&gt;&lt;li&gt;Fine-tuning and post-training of language models for operational use cases&lt;/li&gt;&lt;li&gt;Evaluation frameworks, AI observability and production benchmarking&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;&lt;strong&gt;What you will need&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Degree in Computer Science, Machine Learning, Mathematics or similar, or equivalent demonstrated experience&lt;/li&gt;&lt;li&gt;Around three years or more of professional AI/ML engineering experience&lt;/li&gt;&lt;li&gt;Strong Python, with solid fundamentals across testing, version control and CI/CD&lt;/li&gt;&lt;li&gt;Hands-on experience taking LLM APIs into production, not just prototypes&lt;/li&gt;&lt;li&gt;Familiarity with agentic concepts such as tool and function calling, and agent frameworks&lt;/li&gt;&lt;li&gt;Daily use of AI-assisted coding tools&lt;/li&gt;&lt;li&gt;Ability to read ML research and turn it into practical experiments&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Nice to have&lt;/strong&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;LangGraph, LangChain or similar agent frameworks, MCP a plus&lt;/li&gt;&lt;li&gt;Time-series forecasting and anomaly prediction&lt;/li&gt;&lt;li&gt;Fine-tuning or post-training experience&lt;/li&gt;&lt;li&gt;PyTorch and model serving frameworks&lt;/li&gt;&lt;li&gt;Cloud ML platforms, GCP in particular&lt;/li&gt;&lt;li&gt;LLM evaluation and benchmarking, harness design&lt;/li&gt;&lt;li&gt;Exposure to industrial or building control systems&lt;/li&gt;&lt;li&gt;Background in DevOps, distributed systems or observability tooling&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;&lt;strong&gt;On offer&lt;/strong&gt;&lt;/p&gt;&lt;p&gt;$140,000 to $160,000 base, stock options, full medical, dental and vision, 401(k) and paid time off.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>$140,000.00/yr - $160,000.00/yr</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+AI Engineer (LLM / Agentic Systems)
+Bay Area, California | Hybrid | $140,000 to $160,000 + equity
+A well-funded early stage company is applying AI to the operational side of critical infrastructure. Their platform pulls live data from sensor and control networks across large facilities, then uses agentic AI to spot problems, connect related events and give operators recommendations in real time. It is a genuinely hard technical problem in a market that is growing quickly.
+This suits an engineer with roughly three to six years behind them who has already shipped LLM-powered systems into production and wants more ownership than a large team allows. You would be joining a small engineering group and working end to end, from data pipelines and model integration through to agentic orchestration, evaluation and production support.
+It is not a research role, but research thinking matters. You will be expected to keep up with the field, bring ideas forward and then build them properly.
+What you will work on
+- Multi-agent orchestration and LLM-driven triage workflows
+- Time-series modelling for anomaly detection and failure prediction on multivariate data
+- Retrieval-augmented knowledge systems for operations teams
+- Data and ML pipelines: ingestion, ETL and dataset construction
+- Fine-tuning and post-training of language models for operational use cases
+- Evaluation frameworks, AI observability and production benchmarking
+What you will need
+- Degree in Computer Science, Machine Learning, Mathematics or similar, or equivalent demonstrated experience
+- Around three years or more of professional AI/ML engineering experience
+- Strong Python, with solid fundamentals across testing, version control and CI/CD
+- Hands-on experience taking LLM APIs into production, not just prototypes
+- Familiarity with agentic concepts such as tool and function calling, and agent frameworks
+- Daily use of AI-assisted coding tools
+- Ability to read ML research and turn it into practical experiments
+Nice to have
+- LangGraph, LangChain or similar agent frameworks, MCP a plus
+- Time-series forecasting and anomaly prediction
+- Fine-tuning or post-training experience
+- PyTorch and model serving frameworks
+- Cloud ML platforms, GCP in particular
+- LLM evaluation and benchmarking, harness design
+- Exposure to industrial or building control systems
+- Background in DevOps, distributed systems or observability tooling
+On offer
+$140,000 to $160,000 base, stock options, full medical, dental and vision, 401(k) and paid time off.</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Associate</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>Engineering and Information Technology</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>IT Services and IT Consulting and Data Infrastructure and Analytics</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?position=1&amp;pageNum=0&amp;keywords=AI+Engineer&amp;location=United+States&amp;distance=0&amp;f_TPR=r86400</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr"/>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>http://www.auxotalent.com</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>Auxo is a global STEMx workforce solutions partner, supporting the industries shaping the future of work. We bring together four specialist divisions across Technology, Advanced Engineering, Future Build and Frontier, connecting ambitious organisations with the talent and capability they need to grow.
+Our work spans permanent hiring, contract recruitment, executive search, global mobility, advisory services and complex workforce programmes delivered through Auxo XPO. This unified approach gives clients a single partner with deep expertise, wider reach and stronger delivery across fast changing markets.
+Auxo exists to help businesses stay competitive in a world where skills, industries and technologies evolve quickly. By combining specialist insight with global scale, we help clients build teams that drive progress. For candidates, we open doors to opportunities in the industries that will define tomorrow.
+Challenge. Growth. Tenacity. These values guide how we work and how we deliver for the people and organisations who trust us.
+The future, powered by talent.</t>
+        </is>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>963</t>
+        </is>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>2026-08-14 05:10:51</t>
+        </is>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>Ethan Boon</t>
+        </is>
+      </c>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>Headhunter | Physical AI | Building teams that build robots | Irish | Arsenal Supporter in Manchester</t>
+        </is>
+      </c>
+      <c r="AE28" t="inlineStr">
+        <is>
+          <t>https://media.licdn.com/dms/image/v2/D4E03AQHF_BaaRyQHNw/profile-displayphoto-shrink_400_400/B4EZVhGcC7GgAk-/0/1741090833998?e=2147483647&amp;v=beta&amp;t=W_SUFUWY-1VlSbEteeLD647I3E86TyzrnymebAnwXAI</t>
+        </is>
+      </c>
+      <c r="AF28" t="inlineStr">
+        <is>
+          <t>https://uk.linkedin.com/in/ethan-boon</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>4454092284</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Rwjy3v4AiuPueetqlRJssA==</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Hqan1SC6SBVwlDMjIWeHxQ==</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/ai-engineer-at-translucent-ai-4454092284?position=1&amp;pageNum=0&amp;refId=Hqan1SC6SBVwlDMjIWeHxQ%3D%3D&amp;trackingId=Rwjy3v4AiuPueetqlRJssA%3D%3D</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Translucent AI</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/translucentai?trk=public_jobs_jserp-result_job-search-card-subtitle</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://media.licdn.com/dms/image/v2/D4D0BAQFvaeCnyJlj3Q/company-logo_100_100/B4DZf1jNi_GYAQ-/0/1752171338278/translucentai_logo?e=2147483647&amp;v=beta&amp;t=m775Vd5YtG6VtIENnI4-FaRRYZsVEIxuc-SI6jq8T8w</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>&lt;strong&gt;Role Details&lt;br&gt;&lt;br&gt;&lt;/strong&gt;&lt;ul&gt;&lt;li&gt;Full-Time&lt;/li&gt;&lt;li&gt;Office Location - New York City (hybrid)&lt;br&gt;&lt;br&gt;&lt;/li&gt;&lt;/ul&gt;&lt;strong&gt;Why Translucent&lt;br&gt;&lt;br&gt;&lt;/strong&gt;Healthcare providers drive $2.5 trillion in medical expenditures annually — and operate on razor-thin 2–5% margins. Despite these stakes, the finance teams behind these organizations are buried in spreadsheets, manual data pulls, and disconnected systems, spending more time finding and cleaning data than actually using it to make decisions.&lt;br&gt;&lt;br&gt;Translucent is changing that. We're building the agentic AI platform designed exclusively for healthcare finance— giving every finance team, department, service line their own arsenal of AI Agents that run 24/7, understand their specific data, business logic, and workflows.&lt;br&gt;&lt;br&gt;Founded in 2024 and backed by GV, NEA, FPV, and Virtue, we've already been deployed by healthcare organizations managing over $5 billion in combined revenue. The product-market fit is real, the problem is massive, and we're just getting started. If you want to work at the intersection of AI and one of the most complex, consequential industries in the world, this is the place.&lt;br&gt;&lt;br&gt;&lt;strong&gt;Role Overview&lt;br&gt;&lt;br&gt;&lt;/strong&gt;We're looking for an AI Engineer to help build the agentic platform at the core of Translucent: the AI financial platform transforming how healthcare organizations make business decisions.&lt;br&gt;&lt;br&gt;You'll work hands-on across R&amp;amp;D and platform engineering — improving the underlying agent capabilities every team builds on, rather than configuring agents for a single customer. You'll standardize the tool surfaces new capabilities plug into, make the agent platform ready to integrate across products, and own the evals, context, and harness engineering that make it reliable enough for healthcare finance. You'll match the right agentic architecture to each use case, turn core capabilities into an ecosystem others build on, and own quality end-to-end.&lt;br&gt;&lt;br&gt;If you are energized by fast-paced environments, love sweating the details of production AI systems, partnering closely with product and design, and seeing your work in customers' hands quickly, you'll feel at home here.&lt;br&gt;&lt;br&gt;&lt;strong&gt;What You’ll Do&lt;br&gt;&lt;br&gt;&lt;/strong&gt;&lt;ul&gt;&lt;li&gt;Standardize tool and skill surfaces — define the contracts (MCP-style tool, connector, and skill interfaces) that let us add new capabilities continuously without destabilizing the platform as it grows&lt;/li&gt;&lt;li&gt;Make the agent platform integration-ready — build the connective tissue so agents, tools, context, and data compose cleanly across products, and match the right agentic architecture to each use case&lt;/li&gt;&lt;li&gt;Own evals and benchmarks — build production-grade eval harnesses, replay, and benchmarks for agentic AI, and gate releases on them; in healthcare finance, accuracy is non-negotiable&lt;/li&gt;&lt;li&gt;Lead context and harness engineering — establish best practices for grounding agents in each customer's business rules and data, and for the control loops that keep outputs reliable&lt;/li&gt;&lt;li&gt;Fine-tune and evaluate models — fine-tune in-house and open-source models, benchmark them against frontier baselines, and make the build-vs-buy calls on model, framework, and infra&lt;/li&gt;&lt;li&gt;Turn capabilities into an ecosystem — build reusable core capabilities that translate across features and products, and ship them end-to-end with product and design&lt;br&gt;&lt;br&gt;&lt;/li&gt;&lt;/ul&gt;&lt;strong&gt;What You Have&lt;br&gt;&lt;br&gt;&lt;/strong&gt;&lt;ul&gt;&lt;li&gt;3+ years of software engineering experience, with meaningful production work in Python&lt;/li&gt;&lt;li&gt;Direct experience shipping LLM-powered or agentic systems in production — not just prototypes. You know where models fail and how to make them reliable&lt;/li&gt;&lt;li&gt;Hands-on experience with at least one modern agent framework (LangGraph, Google ADK, LlamaIndex, Claude Agent SDK, or equivalent), and a clear point of view on what to use vs. build&lt;/li&gt;&lt;li&gt;Production evals and benchmarking — you've built eval harnesses and benchmarks that gate real releases, not one-off spot checks&lt;/li&gt;&lt;li&gt;Context engineering — grounding agents through retrieval, context layers, and knowledge transfer so outputs match a specific org or user&lt;/li&gt;&lt;li&gt;Comfort with the data and retrieval layer — SQL, BigQuery or a comparable warehouse, embeddings, and vector search&lt;/li&gt;&lt;li&gt;A bias toward shipping — you take an ambiguous problem to a working V1 fast, then iterate&lt;br&gt;&lt;br&gt;&lt;/li&gt;&lt;/ul&gt;&lt;strong&gt;Plus deep, demonstrable expertise in at least one (ideally two) of the following:&lt;br&gt;&lt;br&gt;&lt;/strong&gt;&lt;ul&gt;&lt;li&gt;Tool-surface and connector platform engineering — standardized tool/skill contracts (e.g., MCP) and connector ecosystems that scale without breaking&lt;/li&gt;&lt;li&gt;Harness and loop engineering — agent control loops, orchestration, and inference harnesses; right-sizing agent architecture per use case and keeping it reliable at scale&lt;/li&gt;&lt;li&gt;Open-source and in-house model fine-tuning — fine-tuning open models and benchmarking them against frontier baselines&lt;/li&gt;&lt;li&gt;Production context-layer engineering — systems that capture business rules and preferences and feed them to agents reliably&lt;br&gt;&lt;br&gt;&lt;/li&gt;&lt;/ul&gt;&lt;strong&gt;Nice to Have&lt;br&gt;&lt;br&gt;&lt;/strong&gt;&lt;ul&gt;&lt;li&gt;Experience with healthcare finance, accounting, or other structured financial data — or genuine curiosity about it&lt;/li&gt;&lt;li&gt;Applied ML or model-evaluation research background&lt;/li&gt;&lt;li&gt;Open-source contributions to agent or LLM tooling&lt;/li&gt;&lt;li&gt;Experience designing tool-use APIs or developer-facing AI products&lt;/li&gt;&lt;li&gt;Familiarity with our stack: Vertex AI (Gemini, Claude on Vertex), GenKit, MCP, BigQuery&lt;br&gt;&lt;br&gt;&lt;/li&gt;&lt;/ul&gt;&lt;strong&gt;Experience Level&lt;br&gt;&lt;br&gt;&lt;/strong&gt;We're looking for engineers who own meaningful surface area and drive work forward independently. You'll bring sharp judgment on architecture and build-vs-buy trade-offs under ambiguity, a bias toward shipping a working V1 fast, and the craft to make agentic systems reliable enough for healthcare finance — not just demos.&lt;br&gt;&lt;br&gt;https://www.translucent.co/&lt;br&gt;&lt;br&gt;&lt;strong&gt;Base Salary&lt;/strong&gt;: $175,000-$275,000 USD + equity</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Role Details
+- Full-Time
+- Office Location - New York City (hybrid)
+Why Translucent
+Healthcare providers drive $2.5 trillion in medical expenditures annually — and operate on razor-thin 2–5% margins. Despite these stakes, the finance teams behind these organizations are buried in spreadsheets, manual data pulls, and disconnected systems, spending more time finding and cleaning data than actually using it to make decisions.
+Translucent is changing that. We're building the agentic AI platform designed exclusively for healthcare finance— giving every finance team, department, service line their own arsenal of AI Agents that run 24/7, understand their specific data, business logic, and workflows.
+Founded in 2024 and backed by GV, NEA, FPV, and Virtue, we've already been deployed by healthcare organizations managing over $5 billion in combined revenue. The product-market fit is real, the problem is massive, and we're just getting started. If you want to work at the intersection of AI and one of the most complex, consequential industries in the world, this is the place.
+Role Overview
+We're looking for an AI Engineer to help build the agentic platform at the core of Translucent: the AI financial platform transforming how healthcare organizations make business decisions.
+You'll work hands-on across R&amp;amp;D and platform engineering — improving the underlying agent capabilities every team builds on, rather than configuring agents for a single customer. You'll standardize the tool surfaces new capabilities plug into, make the agent platform ready to integrate across products, and own the evals, context, and harness engineering that make it reliable enough for healthcare finance. You'll match the right agentic architecture to each use case, turn core capabilities into an ecosystem others build on, and own quality end-to-end.
+If you are energized by fast-paced environments, love sweating the details of production AI systems, partnering closely with product and design, and seeing your work in customers' hands quickly, you'll feel at home here.
+What You’ll Do
+- Standardize tool and skill surfaces — define the contracts (MCP-style tool, connector, and skill interfaces) that let us add new capabilities continuously without destabilizing the platform as it grows
+- Make the agent platform integration-ready — build the connective tissue so agents, tools, context, and data compose cleanly across products, and match the right agentic architecture to each use case
+- Own evals and benchmarks — build production-grade eval harnesses, replay, and benchmarks for agentic AI, and gate releases on them; in healthcare finance, accuracy is non-negotiable
+- Lead context and harness engineering — establish best practices for grounding agents in each customer's business rules and data, and for the control loops that keep outputs reliable
+- Fine-tune and evaluate models — fine-tune in-house and open-source models, benchmark them against frontier baselines, and make the build-vs-buy calls on model, framework, and infra
+- Turn capabilities into an ecosystem — build reusable core capabilities that translate across features and products, and ship them end-to-end with product and design
+What You Have
+- 3+ years of software engineering experience, with meaningful production work in Python
+- Direct experience shipping LLM-powered or agentic systems in production — not just prototypes. You know where models fail and how to make them reliable
+- Hands-on experience with at least one modern agent framework (LangGraph, Google ADK, LlamaIndex, Claude Agent SDK, or equivalent), and a clear point of view on what to use vs. build
+- Production evals and benchmarking — you've built eval harnesses and benchmarks that gate real releases, not one-off spot checks
+- Context engineering — grounding agents through retrieval, context layers, and knowledge transfer so outputs match a specific org or user
+- Comfort with the data and retrieval layer — SQL, BigQuery or a comparable warehouse, embeddings, and vector search
+- A bias toward shipping — you take an ambiguous problem to a working V1 fast, then iterate
+Plus deep, demonstrable expertise in at least one (ideally two) of the following:
+- Tool-surface and connector platform engineering — standardized tool/skill contracts (e.g., MCP) and connector ecosystems that scale without breaking
+- Harness and loop engineering — agent control loops, orchestration, and inference harnesses; right-sizing agent architecture per use case and keeping it reliable at scale
+- Open-source and in-house model fine-tuning — fine-tuning open models and benchmarking them against frontier baselines
+- Production context-layer engineering — systems that capture business rules and preferences and feed them to agents reliably
+Nice to Have
+- Experience with healthcare finance, accounting, or other structured financial data — or genuine curiosity about it
+- Applied ML or model-evaluation research background
+- Open-source contributions to agent or LLM tooling
+- Experience designing tool-use APIs or developer-facing AI products
+- Familiarity with our stack: Vertex AI (Gemini, Claude on Vertex), GenKit, MCP, BigQuery
+Experience Level
+We're looking for engineers who own meaningful surface area and drive work forward independently. You'll bring sharp judgment on architecture and build-vs-buy trade-offs under ambiguity, a bias toward shipping a working V1 fast, and the craft to make agentic systems reliable enough for healthcare finance — not just demos.
+https://www.translucent.co/
+Base Salary: $175,000-$275,000 USD + equity</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>Hospitals and Health Care</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?position=1&amp;pageNum=0&amp;keywords=AI+Engineer&amp;location=United+States&amp;distance=0&amp;f_TPR=r86400</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>{'type': 'PostalAddress', 'addressLocality': 'New York', 'addressRegion': 'New York', 'postalCode': '10003', 'addressCountry': 'US'}</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>https://www.translucent.ai</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>The AI-native platform for healthcare finance.</t>
+        </is>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>Hospitals and clinics shouldn't have to choose between financial health and patient health. But today, they do.
+Healthcare finance teams are drowning in manual data work—pulling numbers from multiple systems, building spreadsheets, answering endless questions from operators. By the time they finish analyzing last month's performance, they're already behind on this month's decisions.
+The result? Finance leaders are forced to make difficult tradeoffs: cut services to stay solvent, or keep services running and risk financial instability.
+What We Do
+Translucent is healthcare's financial operating system. We automate the manual data work that consumes finance teams—connecting fragmented data sources, running analyses, and surfacing insights instantly.
+Instead of spending days building reports, finance teams can focus on what matters: moving the margin and making strategic decisions that improve both financial performance and patient care.
+Why It Matters
+When healthcare finance teams have the financial clarity they need, hospitals can maintain strong margins while delivering excellent patient care. No more forced tradeoffs between the two.
+We serve health systems and medical groups across the United States—from large multi-billion dollar organizations to small rural hospitals where every decision affects whether patients can access care locally.
+Our Team &amp; Backing
+Translucent is backed by GV, NEA, FPV Ventures, Virtue, and Redesign Health. We're headquartered in New York City and bring together expertise in agentic AI, healthcare operations, and enterprise software.</t>
+        </is>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>2026-08-14 05:10:51</t>
+        </is>
+      </c>
+      <c r="AC29" t="inlineStr"/>
+      <c r="AD29" t="inlineStr"/>
+      <c r="AE29" t="inlineStr"/>
+      <c r="AF29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>4454317490</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>iePAq0f204NqU2YILM222w==</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Hqan1SC6SBVwlDMjIWeHxQ==</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/ai-ml-engineer-at-capgemini-4454317490?position=3&amp;pageNum=0&amp;refId=Hqan1SC6SBVwlDMjIWeHxQ%3D%3D&amp;trackingId=iePAq0f204NqU2YILM222w%3D%3D</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>AI/ML Engineer</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Capgemini</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/company/capgemini?trk=public_jobs_jserp-result_job-search-card-subtitle</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>https://media.licdn.com/dms/image/v2/D4E0BAQHIL3HctxNfvg/company-logo_100_100/B4EZokv7VQIUAQ-/0/1761553135376/capgemini_logo?e=2147483647&amp;v=beta&amp;t=zG4Rnn4ZR9lwfNpFaLXXm6DKX3XwtS0cYTIC2dDtWfg</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Atlanta, GA</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Choosing Capgemini means choosing a company where you will be empowered to shape your career in the way you’d like, where you’ll be supported and inspired by a collaborative community of colleagues around the world, and where you’ll be able to reimagine what’s possible. Join us and help the world’s leading organizations unlock the value of technology and build a more sustainable, more inclusive world.&lt;br&gt;&lt;br&gt;&lt;strong&gt;Job Location: Atlanta, GA/ NYC, NY&lt;br&gt;&lt;br&gt;&lt;/strong&gt;&lt;strong&gt;Responsibilities&lt;br&gt;&lt;br&gt;&lt;/strong&gt;We are seeking a highly skilled AIML Engineer with strong hands‑on experience in Python, modern AI/LLM integration, API development, and distributed data technologies.&lt;br&gt;&lt;br&gt;This role will focus on building, integrating, and deploying AI/ML models-particularly those involving Large Language Models (LLMs), agentic AI workflows, and real‑time data pipelines.&lt;br&gt;&lt;br&gt;The ideal candidate will have a strong engineering background with a deep understanding of ML systems design, inferencing pipelines, and microservices‑based APIs.&lt;br&gt;&lt;br&gt;Experience working in Agile environments and collaborating with cross‑functional teams is essential.&lt;br&gt;&lt;br&gt;&lt;strong&gt;Required Skills&lt;br&gt;&lt;br&gt;&lt;/strong&gt;Python&lt;br&gt;&lt;br&gt;Experience in Integration LLM&lt;br&gt;&lt;br&gt;FAST API&lt;br&gt;&lt;br&gt;Kafka Integration&lt;br&gt;&lt;br&gt;Rest API Integration for ML Models&lt;br&gt;&lt;br&gt;GitHub and CoPilot&lt;br&gt;&lt;br&gt;Agentic AI Implementation&lt;br&gt;&lt;br&gt;&lt;strong&gt;Good‑to‑Have Skills&lt;br&gt;&lt;br&gt;&lt;/strong&gt;Java/Angular&lt;br&gt;&lt;br&gt;Spring Boot&lt;br&gt;&lt;br&gt;CI/CD&lt;br&gt;&lt;br&gt;Containerization (Docket, Kubernetes)&lt;br&gt;&lt;br&gt;Cloud ML platforms&lt;br&gt;&lt;br&gt;Finance domain Experience&lt;br&gt;&lt;br&gt;&lt;strong&gt;Life at Capgemini&lt;br&gt;&lt;br&gt;&lt;/strong&gt;Capgemini supports all aspects of your well-being throughout the changing stages of your life and career. For eligible employees, we offer:&lt;br&gt;&lt;br&gt;Flexible work&lt;br&gt;&lt;br&gt;Healthcare including dental, vision, mental health, and well-being programs&lt;br&gt;&lt;br&gt;Financial well-being programs such as 401(k) and Employee Share Ownership Plan&lt;br&gt;&lt;br&gt;Paid time off and paid holidays&lt;br&gt;&lt;br&gt;Paid parental leave&lt;br&gt;&lt;br&gt;Family building benefits like adoption assistance, surrogacy, and cryopreservation&lt;br&gt;&lt;br&gt;Social well-being benefits like subsidized back-up child/elder care and tutoring&lt;br&gt;&lt;br&gt;Mentoring, coaching and learning programs&lt;br&gt;&lt;br&gt;Employee Resource Groups nd Qualifications required for this position. Physical, mental, sensory or environmental demands may be referenced in an attempt to communicate the manner in which this position traditionally is performed. Whenever necessary to provide individuals with disabilities an equal employment opportunity, Capgemini will consider reasonable accommodations that might involve varying job requirements and/or changing the way this job is performed, provided that such accommodations do not pose an undue hardship.&lt;br&gt;&lt;br&gt;Capgemini is committed to providing reasonable accommodations&lt;br&gt;&lt;br&gt;Disaster Relief&lt;br&gt;&lt;br&gt;The base compensation range for this role in the posted location is: 103330 to 128656&lt;br&gt;&lt;br&gt;Capgemini provides compensation range information in accordance with applicable national, state, provincial, and local pay transparency laws. The base compensation range listed for this position reflects the minimum and maximum target compensation Capgemini, in good faith, believes it may pay for the role at the time of this posting. This range may be subject to change as permitted by law.&lt;br&gt;&lt;br&gt;The actual compensation offered to any candidate may fall outside of the posted range and will be determined based on multiple factors legally permitted in the applicable jurisdiction.&lt;br&gt;&lt;br&gt;These may include, but are not limited to: Geographic location, Education and qualifications, Certifications and licenses, Relevant experience and skills, Seniority and performance, Market and business consideration, Internal pay equity.&lt;br&gt;&lt;br&gt;It is not typical for candidates to be hired at or near the top of the posted compensation range.&lt;br&gt;&lt;br&gt;In addition to base salary, this role may be eligible for additional compensation such as variable incentives, bonuses, or commissions, depending on the position and applicable laws.&lt;br&gt;&lt;br&gt;&lt;strong&gt;Capgemini offers a comprehensive, non-negotiable benefits package to all regular, full-time employees.&lt;/strong&gt; In the U.S. and Canada, available benefits are determined by local policy and eligibility and may include:&lt;br&gt;&lt;br&gt;&lt;ul&gt;&lt;li&gt;Paid time off based on employee grade (A-F), defined by policy: Vacation: 12-25 days, depending on grade, Company paid holidays, Personal Days, Sick Leave&lt;/li&gt;&lt;li&gt;Medical, dental, and vision coverage (or provincial healthcare coordination in Canada)&lt;/li&gt;&lt;li&gt;Retirement savings plans (e.g., 401(k) in the U.S., RRSP in Canada)&lt;/li&gt;&lt;li&gt;Life and disability insurance&lt;/li&gt;&lt;li&gt;Employee assistance programs&lt;/li&gt;&lt;li&gt;Other benefits as provided by local policy and eligibility&lt;br&gt;&lt;br&gt;&lt;/li&gt;&lt;/ul&gt;&lt;strong&gt;Important Notice:&lt;/strong&gt; Compensation (including bonuses, commissions, or other forms of incentive pay) is not considered earned, vested, or payable until it becomes due under the terms of applicable plans or agreements and is subject to Capgemini’s discretion, consistent with applicable laws. The Company reserves the right to amend or withdraw compensation programs at any time, within the limits of applicable legislation.&lt;br&gt;&lt;br&gt;&lt;strong&gt;Disclaimers&lt;br&gt;&lt;br&gt;&lt;/strong&gt;Capgemini is an Equal Opportunity Employer encouraging inclusion in the workplace. Capgemini also participates in the Partnership Accreditation in Indigenous Relations (PAIR) program which supports meaningful engagement with Indigenous communities across Canada by promoting fairness, accessibility, inclusion and respect. We value the rich cultural heritage and contributions of Indigenous Peoples and actively work to create a welcoming and respectful environment. All qualified applicants will receive consideration for employment without regard to race, national origin, gender identity/expression, age, religion, disability, sexual orientation, genetics, veteran status, marital status or any other characteristic protected by law.&lt;br&gt;&lt;br&gt;This is a general description of the Duties, Responsibilities and Qualifications required for this position. Physical, mental, sensory or environmental demands may be referenced in an attempt to communicate the manner in which this position traditionally is performed. Whenever necessary to provide individuals with disabilities an equal employment opportunity, Capgemini will consider reasonable accommodations that might involve varying job requirements and/or changing the way this job is performed, provided that such accommodation does not pose an undue hardship. Capgemini is committed to providing reasonable accommodation during our recruitment process. If you need assistance or accommodation, please reach out to your recruiting contact.&lt;br&gt;&lt;br&gt;Please be aware that Capgemini may capture your image (video or screenshot) during the interview process and that image may be used for verification, including during the hiring and onboarding process.&lt;br&gt;&lt;br&gt;Click the following link for more information on your rights as an Applicant in the United States. http://www.capgemini.com/resources/equal-employment-opportunity-is-the-law&lt;br&gt;&lt;br&gt;Capgemini is a global business and technology transformation partner, helping organizations to accelerate their dual transition to a digital and sustainable world, while creating tangible impact for enterprises and society. It is a responsible and diverse group of 340,000 team members in more than 50 countries. With its strong over 55-year heritage, Capgemini is trusted by its clients to unlock the value of technology to address the entire breadth of their business needs. It delivers end-to-end services and solutions leveraging strengths from strategy and design to engineering, all fueled by its market leading capabilities in AI, generative AI, cloud and data, combined with its deep industry expertise and partner ecosystem.</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Choosing Capgemini means choosing a company where you will be empowered to shape your career in the way you’d like, where you’ll be supported and inspired by a collaborative community of colleagues around the world, and where you’ll be able to reimagine what’s possible. Join us and help the world’s leading organizations unlock the value of technology and build a more sustainable, more inclusive world.
+Job Location: Atlanta, GA/ NYC, NY
+Responsibilities
+We are seeking a highly skilled AIML Engineer with strong hands‑on experience in Python, modern AI/LLM integration, API development, and distributed data technologies.
+This role will focus on building, integrating, and deploying AI/ML models-particularly those involving Large Language Models (LLMs), agentic AI workflows, and real‑time data pipelines.
+The ideal candidate will have a strong engineering background with a deep understanding of ML systems design, inferencing pipelines, and microservices‑based APIs.
+Experience working in Agile environments and collaborating with cross‑functional teams is essential.
+Required Skills
+Python
+Experience in Integration LLM
+FAST API
+Kafka Integration
+Rest API Integration for ML Models
+GitHub and CoPilot
+Agentic AI Implementation
+Good‑to‑Have Skills
+Java/Angular
+Spring Boot
+CI/CD
+Containerization (Docket, Kubernetes)
+Cloud ML platforms
+Finance domain Experience
+Life at Capgemini
+Capgemini supports all aspects of your well-being throughout the changing stages of your life and career. For eligible employees, we offer:
+Flexible work
+Healthcare including dental, vision, mental health, and well-being programs
+Financial well-being programs such as 401(k) and Employee Share Ownership Plan
+Paid time off and paid holidays
+Paid parental leave
+Family building benefits like adoption assistance, surrogacy, and cryopreservation
+Social well-being benefits like subsidized back-up child/elder care and tutoring
+Mentoring, coaching and learning programs
+Employee Resource Groups nd Qualifications required for this position. Physical, mental, sensory or environmental demands may be referenced in an attempt to communicate the manner in which this position traditionally is performed. Whenever necessary to provide individuals with disabilities an equal employment opportunity, Capgemini will consider reasonable accommodations that might involve varying job requirements and/or changing the way this job is performed, provided that such accommodations do not pose an undue hardship.
+Capgemini is committed to providing reasonable accommodations
+Disaster Relief
+The base compensation range for this role in the posted location is: 103330 to 128656
+Capgemini provides compensation range information in accordance with applicable national, state, provincial, and local pay transparency laws. The base compensation range listed for this position reflects the minimum and maximum target compensation Capgemini, in good faith, believes it may pay for the role at the time of this posting. This range may be subject to change as permitted by law.
+The actual compensation offered to any candidate may fall outside of the posted range and will be determined based on multiple factors legally permitted in the applicable jurisdiction.
+These may include, but are not limited to: Geographic location, Education and qualifications, Certifications and licenses, Relevant experience and skills, Seniority and performance, Market and business consideration, Internal pay equity.
+It is not typical for candidates to be hired at or near the top of the posted compensation range.
+In addition to base salary, this role may be eligible for additional compensation such as variable incentives, bonuses, or commissions, depending on the position and applicable laws.
+Capgemini offers a comprehensive, non-negotiable benefits package to all regular, full-time employees. In the U.S. and Canada, available benefits are determined by local policy and eligibility and may include:
+- Paid time off based on employee grade (A-F), defined by policy: Vacation: 12-25 days, depending on grade, Company paid holidays, Personal Days, Sick Leave
+- Medical, dental, and vision coverage (or provincial healthcare coordination in Canada)
+- Retirement savings plans (e.g., 401(k) in the U.S., RRSP in Canada)
+- Life and disability insurance
+- Employee assistance programs
+- Other benefits as provided by local policy and eligibility
+Important Notice: Compensation (including bonuses, commissions, or other forms of incentive pay) is not considered earned, vested, or payable until it becomes due under the terms of applicable plans or agreements and is subject to Capgemini’s discretion, consistent with applicable laws. The Company reserves the right to amend or withdraw compensation programs at any time, within the limits of applicable legislation.
+Disclaimers
+Capgemini is an Equal Opportunity Employer encouraging inclusion in the workplace. Capgemini also participates in the Partnership Accreditation in Indigenous Relations (PAIR) program which supports meaningful engagement with Indigenous communities across Canada by promoting fairness, accessibility, inclusion and respect. We value the rich cultural heritage and contributions of Indigenous Peoples and actively work to create a welcoming and respectful environment. All qualified applicants will receive consideration for employment without regard to race, national origin, gender identity/expression, age, religion, disability, sexual orientation, genetics, veteran status, marital status or any other characteristic protected by law.
+This is a general description of the Duties, Responsibilities and Qualifications required for this position. Physical, mental, sensory or environmental demands may be referenced in an attempt to communicate the manner in which this position traditionally is performed. Whenever necessary to provide individuals with disabilities an equal employment opportunity, Capgemini will consider reasonable accommodations that might involve varying job requirements and/or changing the way this job is performed, provided that such accommodation does not pose an undue hardship. Capgemini is committed to providing reasonable accommodation during our recruitment process. If you need assistance or accommodation, please reach out to your recruiting contact.
+Please be aware that Capgemini may capture your image (video or screenshot) during the interview process and that image may be used for verification, including during the hiring and onboarding process.
+Click the following link for more information on your rights as an Applicant in the United States. http://www.capgemini.com/resources/equal-employment-opportunity-is-the-law
+Capgemini is a global business and technology transformation partner, helping organizations to accelerate their dual transition to a digital and sustainable world, while creating tangible impact for enterprises and society. It is a responsible and diverse group of 340,000 team members in more than 50 countries. With its strong over 55-year heritage, Capgemini is trusted by its clients to unlock the value of technology to address the entire breadth of their business needs. It delivers end-to-end services and solutions leveraging strengths from strategy and design to engineering, all fueled by its market leading capabilities in AI, generative AI, cloud and data, combined with its deep industry expertise and partner ecosystem.</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>Engineering and Information Technology</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>IT Services and IT Consulting</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?position=1&amp;pageNum=0&amp;keywords=AI+Engineer&amp;location=United+States&amp;distance=0&amp;f_TPR=r86400</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>{'type': 'PostalAddress', 'streetAddress': "Place de l'Étoile", 'addressLocality': 'Paris', 'addressRegion': 'France', 'postalCode': '75017', 'addressCountry': 'FR'}</t>
+        </is>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>https://www.capgemini.com</t>
+        </is>
+      </c>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t>Make it real.</t>
+        </is>
+      </c>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Capgemini is an AI-powered global business and technology transformation partner, delivering tangible business value. We imagine the future of organizations and make it real with AI, technology and people. With our strong heritage of nearly 60 years, we are a responsible and diverse group of 420,000 team members in more than 50 countries. We deliver end-to-end services and solutions with our deep industry expertise and strong partner ecosystem, leveraging our capabilities across strategy, technology, design, engineering and business operations. The Group reported 2025 global revenues of €22.5 billion.
+Make it real | www.capgemini.com
+</t>
+        </is>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>347372</t>
+        </is>
+      </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="AB30" t="inlineStr">
+        <is>
+          <t>2026-08-14 05:10:51</t>
+        </is>
+      </c>
+      <c r="AC30" t="inlineStr"/>
+      <c r="AD30" t="inlineStr"/>
+      <c r="AE30" t="inlineStr"/>
+      <c r="AF30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>4454367102</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>AJ+4G+1PpZWM90ASw6AeVw==</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Hqan1SC6SBVwlDMjIWeHxQ==</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/applied-ai-engineer-at-meeboss-4454367102?position=2&amp;pageNum=0&amp;refId=Hqan1SC6SBVwlDMjIWeHxQ%3D%3D&amp;trackingId=AJ%2B4G%2B1PpZWM90ASw6AeVw%3D%3D</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Applied AI Engineer</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>MeeBoss</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/meeboss?trk=public_jobs_jserp-result_job-search-card-subtitle</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://media.licdn.com/dms/image/v2/D560BAQH7KwZNWpOqRg/company-logo_100_100/B56ZcuuX28GsAQ-/0/1748835598284/meeboss_logo?e=2147483647&amp;v=beta&amp;t=kIyFeq5olRjgZVEaLtZYV4GgvbbKxUxoI-Xw6gtzuHY</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;About the job&lt;/strong&gt;&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;MeeBoss is sharing this active opportunity on behalf of the hiring company. This role involves building systems that automate finance operations by deploying AI to operate computers like humans, navigating browsers, processing documents, and working through legacy systems for large enterprises.&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;The position focuses on browser agent reliability, document understanding, and inference optimization to improve accuracy and speed.&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Job title&lt;/strong&gt;&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;Applied AI Engineer&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Company&lt;/strong&gt;&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;MeeBoss&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Location&lt;/strong&gt;&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;San Francisco, CA On-site&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;&lt;strong&gt;Compensation&lt;/strong&gt;&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;$180,000-250,000/year&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;&lt;strong&gt;What you will do&lt;/strong&gt;&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Work on browser agent reliability, document understanding, and inference optimization.&lt;/li&gt;&lt;li&gt;Push to state-of-the-art across core automation capabilities including UI interaction, unstructured data parsing, and tool use.&lt;/li&gt;&lt;li&gt;Build adaptive systems that self-heal when environments change.&lt;/li&gt;&lt;li&gt;Design fine-tuning pipelines that learn from customer-specific workflows.&lt;/li&gt;&lt;li&gt;Optimize latency across the stack through model selection, quantization, caching, and routing strategies.&lt;/li&gt;&lt;li&gt;Turn research into production systems.&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;&lt;strong&gt;What we are looking for&lt;/strong&gt;&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;Strong Python expertise and proficiency in ML frameworks, particularly PyTorch.&lt;/li&gt;&lt;li&gt;Eval-and-metric mindset, focusing on production metrics rather than just benchmarks.&lt;/li&gt;&lt;li&gt;Comfort with messy data and the ability to make it useful.&lt;/li&gt;&lt;li&gt;Track record of shipping end-to-end systems.&lt;/li&gt;&lt;li&gt;Clear communication skills to describe work without buzzwords.&lt;/li&gt;&lt;li&gt;Based in San Francisco or willing to relocate for in-person work 5 days a week.&lt;/li&gt;&lt;li&gt;Experience with RL, retrieval systems, or agent-based systems (Nice-to-have).&lt;/li&gt;&lt;li&gt;Cross-stack range including inference optimization, data pipelines, fine-tuning, and model monitoring (Nice-to-have).&lt;/li&gt;&lt;li&gt;Published ML papers or significant OSS contributions (Nice-to-have).&lt;/li&gt;&lt;li&gt;Lab or research exposure (Nice-to-have).&lt;/li&gt;&lt;li&gt;Recent applied work on LLMs, browser agents, RAG, or production AI workflows (Nice-to-have).&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;&lt;strong&gt;About MeeBoss&lt;/strong&gt;&lt;/p&gt;&lt;p&gt;&lt;br&gt;&lt;/p&gt;&lt;p&gt;MeeBoss helps job seekers and hiring teams make direct, relevant career connections.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+About the job
+MeeBoss is sharing this active opportunity on behalf of the hiring company. This role involves building systems that automate finance operations by deploying AI to operate computers like humans, navigating browsers, processing documents, and working through legacy systems for large enterprises.
+The position focuses on browser agent reliability, document understanding, and inference optimization to improve accuracy and speed.
+Job title
+Applied AI Engineer
+Company
+MeeBoss
+Location
+San Francisco, CA On-site
+Compensation
+$180,000-250,000/year
+What you will do
+- Work on browser agent reliability, document understanding, and inference optimization.
+- Push to state-of-the-art across core automation capabilities including UI interaction, unstructured data parsing, and tool use.
+- Build adaptive systems that self-heal when environments change.
+- Design fine-tuning pipelines that learn from customer-specific workflows.
+- Optimize latency across the stack through model selection, quantization, caching, and routing strategies.
+- Turn research into production systems.
+What we are looking for
+- Strong Python expertise and proficiency in ML frameworks, particularly PyTorch.
+- Eval-and-metric mindset, focusing on production metrics rather than just benchmarks.
+- Comfort with messy data and the ability to make it useful.
+- Track record of shipping end-to-end systems.
+- Clear communication skills to describe work without buzzwords.
+- Based in San Francisco or willing to relocate for in-person work 5 days a week.
+- Experience with RL, retrieval systems, or agent-based systems (Nice-to-have).
+- Cross-stack range including inference optimization, data pipelines, fine-tuning, and model monitoring (Nice-to-have).
+- Published ML papers or significant OSS contributions (Nice-to-have).
+- Lab or research exposure (Nice-to-have).
+- Recent applied work on LLMs, browser agents, RAG, or production AI workflows (Nice-to-have).
+About MeeBoss
+MeeBoss helps job seekers and hiring teams make direct, relevant career connections.</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>Mid-Senior level</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>Engineering, Information Technology, and Marketing</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>Human Resources Services</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?position=1&amp;pageNum=0&amp;keywords=AI+Engineer&amp;location=United+States&amp;distance=0&amp;f_TPR=r86400</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>{'type': 'PostalAddress', 'streetAddress': '10800 NE 8th St', 'addressLocality': 'Bellevue', 'addressRegion': 'Washington', 'postalCode': '98004', 'addressCountry': 'US'}</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>meeboss.com</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>We simplify hiring through fast job matching and direct connections, all in one seamless platform.</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>MeeBoss is transforming the hiring experience by building the human connection early. Experience the transformative power of our innovative job-matching and direct chat platform designed to help companies find the right talent faster and more affordably. Personalized matches and direct two-way engagement empowers job seekers and employers to quickly connect, assess fit, and advance the process. Skip the noise – Download MeeBoss today!</t>
+        </is>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>2026-08-14 05:10:51</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>Wenjing Zhou</t>
+        </is>
+      </c>
+      <c r="AD31" t="inlineStr"/>
+      <c r="AE31" t="inlineStr">
+        <is>
+          <t>https://static.licdn.com/aero-v1/sc/h/9c8pery4andzj6ohjkjp54ma2</t>
+        </is>
+      </c>
+      <c r="AF31" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/wenjing-zhou-84a117422</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>